<commit_message>
Działa dobrze wraz z ładowaniem urzędów skarbowych
</commit_message>
<xml_diff>
--- a/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
+++ b/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\AddressLibrary\AddressLibrary\AppData\Dictionaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B4F4BB-E8B3-4A35-88DF-AA8A9ED9FD3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2E0C7B1-AFA6-4801-8821-00A40977B207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="760">
   <si>
     <t>abp</t>
   </si>
@@ -260,9 +260,6 @@
     <t>kpt. cichociemnego</t>
   </si>
   <si>
-    <t>kpt. hcm.</t>
-  </si>
-  <si>
     <t>kpt. pil.</t>
   </si>
   <si>
@@ -2295,6 +2292,30 @@
   </si>
   <si>
     <t>bł. ks. kard. prym.</t>
+  </si>
+  <si>
+    <t>doktora medycyny harcmistrza</t>
+  </si>
+  <si>
+    <t>doktor medycyny harcmistrz</t>
+  </si>
+  <si>
+    <t>dr med. hm.</t>
+  </si>
+  <si>
+    <t>kpt. hm.</t>
+  </si>
+  <si>
+    <t>doktorzy</t>
+  </si>
+  <si>
+    <t>harmistrze</t>
+  </si>
+  <si>
+    <t>doktorów</t>
+  </si>
+  <si>
+    <t>harcmistrzów</t>
   </si>
 </sst>
 </file>
@@ -2667,7 +2688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD74A5C-AF8A-492F-8246-0B7893A73121}">
-  <dimension ref="A1:C286"/>
+  <dimension ref="A1:C289"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" customWidth="1"/>
@@ -2677,21 +2698,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B1" t="s">
         <v>261</v>
       </c>
-      <c r="B1" t="s">
-        <v>262</v>
-      </c>
       <c r="C1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
@@ -2699,10 +2720,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -2710,10 +2731,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -2721,10 +2742,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B5" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -2732,10 +2753,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
@@ -2743,10 +2764,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C7" t="s">
         <v>0</v>
@@ -2754,10 +2775,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -2765,10 +2786,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C9" t="s">
         <v>2</v>
@@ -2776,10 +2797,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
@@ -2787,7 +2808,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B11" t="s">
         <v>8</v>
@@ -2798,7 +2819,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B12" t="s">
         <v>9</v>
@@ -2809,10 +2830,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C13" t="s">
         <v>24</v>
@@ -2820,10 +2841,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C14" t="s">
         <v>10</v>
@@ -2831,10 +2852,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C15" t="s">
         <v>10</v>
@@ -2842,10 +2863,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B16" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C16" t="s">
         <v>14</v>
@@ -2853,10 +2874,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B17" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C17" t="s">
         <v>20</v>
@@ -2864,10 +2885,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C18" t="s">
         <v>22</v>
@@ -2875,10 +2896,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B19" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C19" t="s">
         <v>23</v>
@@ -2886,10 +2907,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="B20" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C20" t="s">
         <v>10</v>
@@ -2897,10 +2918,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B21" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C21" t="s">
         <v>11</v>
@@ -2908,10 +2929,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B22" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -2919,10 +2940,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B23" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C23" t="s">
         <v>13</v>
@@ -2930,10 +2951,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B24" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C24" t="s">
         <v>15</v>
@@ -2941,10 +2962,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B25" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C25" t="s">
         <v>16</v>
@@ -2952,10 +2973,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B26" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C26" t="s">
         <v>17</v>
@@ -2963,10 +2984,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B27" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C27" t="s">
         <v>18</v>
@@ -2974,10 +2995,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B28" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C28" t="s">
         <v>19</v>
@@ -2985,10 +3006,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="B29" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C29" t="s">
         <v>19</v>
@@ -2996,10 +3017,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B30" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C30" t="s">
         <v>21</v>
@@ -3007,10 +3028,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B31" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C31" t="s">
         <v>26</v>
@@ -3018,21 +3039,21 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="C32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B33" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C33" t="s">
         <v>25</v>
@@ -3040,10 +3061,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B34" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C34" t="s">
         <v>27</v>
@@ -3051,10 +3072,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B35" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C35" t="s">
         <v>28</v>
@@ -3062,10 +3083,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B36" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C36" t="s">
         <v>31</v>
@@ -3073,10 +3094,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B37" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C37" t="s">
         <v>32</v>
@@ -3084,10 +3105,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B38" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C38" t="s">
         <v>33</v>
@@ -3095,10 +3116,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B39" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C39" t="s">
         <v>33</v>
@@ -3106,10 +3127,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B40" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C40" t="s">
         <v>34</v>
@@ -3117,10 +3138,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B41" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C41" t="s">
         <v>36</v>
@@ -3128,10 +3149,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B42" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C42" t="s">
         <v>35</v>
@@ -3139,10 +3160,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B43" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C43" t="s">
         <v>37</v>
@@ -3150,10 +3171,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B44" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C44" t="s">
         <v>38</v>
@@ -3161,10 +3182,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B45" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C45" t="s">
         <v>29</v>
@@ -3172,10 +3193,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B46" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C46" t="s">
         <v>30</v>
@@ -3183,10 +3204,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B47" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C47" t="s">
         <v>29</v>
@@ -3194,10 +3215,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="B48" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C48" t="s">
         <v>30</v>
@@ -3205,10 +3226,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="B49" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C49" t="s">
         <v>29</v>
@@ -3216,10 +3237,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B50" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C50" t="s">
         <v>39</v>
@@ -3227,10 +3248,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B51" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C51" t="s">
         <v>40</v>
@@ -3238,10 +3259,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B52" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C52" t="s">
         <v>40</v>
@@ -3249,10 +3270,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B53" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C53" t="s">
         <v>41</v>
@@ -3260,10 +3281,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B54" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C54" t="s">
         <v>42</v>
@@ -3271,10 +3292,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B55" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C55" t="s">
         <v>42</v>
@@ -3282,10 +3303,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B56" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C56" t="s">
         <v>43</v>
@@ -3293,10 +3314,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B57" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C57" t="s">
         <v>44</v>
@@ -3304,10 +3325,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B58" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C58" t="s">
         <v>45</v>
@@ -3315,10 +3336,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B59" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C59" t="s">
         <v>46</v>
@@ -3326,10 +3347,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B60" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C60" t="s">
         <v>47</v>
@@ -3337,10 +3358,10 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B61" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C61" t="s">
         <v>48</v>
@@ -3348,10 +3369,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B62" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C62" t="s">
         <v>50</v>
@@ -3359,10 +3380,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B63" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C63" t="s">
         <v>50</v>
@@ -3370,10 +3391,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B64" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C64" t="s">
         <v>51</v>
@@ -3381,10 +3402,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B65" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="C65" t="s">
         <v>52</v>
@@ -3392,10 +3413,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B66" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C66" t="s">
         <v>52</v>
@@ -3403,10 +3424,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B67" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C67" t="s">
         <v>49</v>
@@ -3414,10 +3435,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B68" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C68" t="s">
         <v>53</v>
@@ -3425,10 +3446,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B69" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C69" t="s">
         <v>53</v>
@@ -3436,10 +3457,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B70" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C70" t="s">
         <v>54</v>
@@ -3447,10 +3468,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B71" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C71" t="s">
         <v>55</v>
@@ -3458,10 +3479,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B72" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C72" t="s">
         <v>56</v>
@@ -3469,10 +3490,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B73" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C73" t="s">
         <v>57</v>
@@ -3480,10 +3501,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B74" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C74" t="s">
         <v>58</v>
@@ -3491,10 +3512,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B75" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C75" t="s">
         <v>61</v>
@@ -3502,10 +3523,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B76" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C76" t="s">
         <v>60</v>
@@ -3513,7 +3534,7 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B77" t="s">
         <v>62</v>
@@ -3524,7 +3545,7 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B78" t="s">
         <v>63</v>
@@ -3535,10 +3556,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B79" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C79" t="s">
         <v>72</v>
@@ -3546,10 +3567,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B80" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C80" t="s">
         <v>73</v>
@@ -3557,54 +3578,54 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B81" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C81" t="s">
-        <v>74</v>
+        <v>755</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B82" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C82" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B83" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C83" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B84" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C84" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B85" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C85" t="s">
         <v>70</v>
@@ -3612,10 +3633,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B86" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C86" t="s">
         <v>71</v>
@@ -3623,10 +3644,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B87" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C87" t="s">
         <v>64</v>
@@ -3634,7 +3655,7 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B88" t="s">
         <v>65</v>
@@ -3645,10 +3666,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B89" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C89" t="s">
         <v>66</v>
@@ -3656,10 +3677,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B90" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C90" t="s">
         <v>68</v>
@@ -3667,10 +3688,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B91" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C91" t="s">
         <v>67</v>
@@ -3678,7 +3699,7 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B92" t="s">
         <v>69</v>
@@ -3689,10 +3710,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B93" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C93" t="s">
         <v>59</v>
@@ -3700,10 +3721,10 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B94" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C94" t="s">
         <v>59</v>
@@ -3711,2114 +3732,2147 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B95" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C95" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B96" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C96" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B97" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C97" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B98" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C98" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B99" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C99" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B100" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C100" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B101" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C101" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B102" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C102" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B103" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C103" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B104" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C104" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B105" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C105" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B106" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C106" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B107" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C107" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B108" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C108" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B109" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C109" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B110" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C110" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B111" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C111" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B112" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C112" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B113" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C113" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B114" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C114" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B115" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C115" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B116" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C116" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B117" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C117" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B118" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C118" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B119" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C119" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B120" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C120" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B121" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C121" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B122" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C122" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B123" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C123" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B124" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C124" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B125" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C125" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B126" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C126" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B127" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C127" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B128" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C128" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
+        <v>557</v>
+      </c>
+      <c r="B129" t="s">
         <v>558</v>
       </c>
-      <c r="B129" t="s">
-        <v>559</v>
-      </c>
       <c r="C129" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B130" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C130" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B131" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C131" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B132" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C132" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B133" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C133" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B134" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C134" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B135" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C135" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B136" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C136" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B137" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C137" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B138" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C138" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B139" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C139" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B140" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C140" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B141" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C141" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B142" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C142" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B143" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C143" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B144" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C144" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B145" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C145" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B146" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C146" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B147" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C147" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B148" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C148" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B149" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C149" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B150" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C150" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B151" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C151" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B152" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C152" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B153" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C153" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B154" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C154" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B155" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C155" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B156" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C156" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B157" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C157" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B158" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C158" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B159" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C159" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B160" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C160" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B161" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C161" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B162" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C162" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B163" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C163" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B164" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C164" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B165" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C165" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B166" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C166" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B167" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C167" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B168" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C168" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B169" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C169" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B170" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C170" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B171" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C171" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B172" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C172" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B173" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C173" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B174" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C174" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B175" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C175" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B176" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C176" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B177" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C177" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B178" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C178" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B179" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C179" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B180" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C180" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B181" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C181" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B182" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C182" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B183" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C183" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B184" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C184" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B185" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C185" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B186" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C186" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B187" t="s">
+        <v>396</v>
+      </c>
+      <c r="C187" t="s">
         <v>397</v>
-      </c>
-      <c r="C187" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B188" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C188" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B189" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C189" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B190" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C190" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B191" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C191" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B192" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C192" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B193" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C193" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B194" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C194" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B195" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C195" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B196" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C196" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B197" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C197" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B198" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C198" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B199" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C199" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B200" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C200" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B201" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C201" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B202" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C202" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B203" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C203" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B204" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C204" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B205" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C205" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B206" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="C206" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B207" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C207" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B208" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C208" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B209" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C209" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B210" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C210" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="B211" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C211" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B212" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C212" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B213" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C213" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B214" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C214" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B215" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C215" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B216" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C216" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B217" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C217" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B218" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C218" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B219" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C219" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B220" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C220" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B221" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C221" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B222" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C222" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B223" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C223" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B224" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C224" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B225" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C225" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B226" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C226" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B227" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C227" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B228" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C228" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B229" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C229" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B230" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C230" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B231" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C231" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B232" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C232" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B233" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C233" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B234" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C234" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B235" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C235" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B236" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C236" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
+        <v>216</v>
+      </c>
+      <c r="B237" t="s">
         <v>217</v>
       </c>
-      <c r="B237" t="s">
-        <v>218</v>
-      </c>
       <c r="C237" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B238" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C238" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B239" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C239" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B240" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C240" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B241" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C241" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B242" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C242" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B243" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C243" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B244" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="C244" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B245" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C245" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B246" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C246" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B247" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C247" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B248" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C248" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B249" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C249" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="B250" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C250" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B251" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C251" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B252" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C252" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B253" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C253" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B254" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C254" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B255" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C255" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B256" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C256" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B257" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C257" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B258" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C258" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B259" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C259" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="B260" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C260" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B261" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C261" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="B262" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C262" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B263" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C263" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
+        <v>684</v>
+      </c>
+      <c r="B264" t="s">
         <v>685</v>
       </c>
-      <c r="B264" t="s">
-        <v>686</v>
-      </c>
       <c r="C264" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B265" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C265" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B266" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C266" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="B267" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C267" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B268" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C268" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B269" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C269" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B270" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C270" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B271" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C271" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
+        <v>741</v>
+      </c>
+      <c r="B272" t="s">
+        <v>714</v>
+      </c>
+      <c r="C272" t="s">
         <v>742</v>
-      </c>
-      <c r="B272" t="s">
-        <v>715</v>
-      </c>
-      <c r="C272" t="s">
-        <v>743</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B273" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="C273" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B274" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="C274" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B275" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="C275" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B276" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="C276" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B277" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="C277" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B278" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="C278" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B279" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C279" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B280" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="C280" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="B281" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="C281" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B282" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="C282" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B283" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="C283" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="B284" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="C284" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B285" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="C285" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="B286" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="C286" t="s">
-        <v>729</v>
+        <v>728</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
+        <v>753</v>
+      </c>
+      <c r="B287" t="s">
+        <v>752</v>
+      </c>
+      <c r="C287" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
+        <v>756</v>
+      </c>
+      <c r="B288" t="s">
+        <v>758</v>
+      </c>
+      <c r="C288" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>757</v>
+      </c>
+      <c r="B289" t="s">
+        <v>759</v>
+      </c>
+      <c r="C289" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Poprawki w excelach. około 30 pozycji w PNA wymaga korekt
</commit_message>
<xml_diff>
--- a/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
+++ b/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\AddressLibrary\AddressLibrary\AppData\Dictionaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9152B11F-A7E9-464B-A150-58CF4BF0B36F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC0592E-21D0-4D0A-B426-C1DD3D07F832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="757">
   <si>
     <t>abp</t>
   </si>
@@ -2301,6 +2301,12 @@
   </si>
   <si>
     <t>pułkownik profesor</t>
+  </si>
+  <si>
+    <t>biskupi</t>
+  </si>
+  <si>
+    <t>biskupów</t>
   </si>
 </sst>
 </file>
@@ -2673,7 +2679,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD74A5C-AF8A-492F-8246-0B7893A73121}">
-  <dimension ref="A1:C286"/>
+  <dimension ref="A1:C287"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" customWidth="1"/>
@@ -2826,21 +2832,21 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>444</v>
+        <v>755</v>
       </c>
       <c r="B14" t="s">
-        <v>259</v>
+        <v>756</v>
       </c>
       <c r="C14" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B15" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C15" t="s">
         <v>10</v>
@@ -2848,255 +2854,255 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
       <c r="B16" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>455</v>
+        <v>448</v>
       </c>
       <c r="B17" t="s">
-        <v>454</v>
+        <v>263</v>
       </c>
       <c r="C17" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B18" t="s">
-        <v>278</v>
+        <v>454</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B19" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>689</v>
+        <v>458</v>
       </c>
       <c r="B20" t="s">
-        <v>679</v>
+        <v>279</v>
       </c>
       <c r="C20" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>445</v>
+        <v>689</v>
       </c>
       <c r="B21" t="s">
-        <v>260</v>
+        <v>679</v>
       </c>
       <c r="C21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B22" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B23" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B24" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C24" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B25" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="C25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="B26" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C26" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>725</v>
+        <v>452</v>
       </c>
       <c r="B27" t="s">
-        <v>700</v>
+        <v>275</v>
       </c>
       <c r="C27" t="s">
-        <v>736</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>453</v>
+        <v>725</v>
       </c>
       <c r="B28" t="s">
-        <v>276</v>
+        <v>700</v>
       </c>
       <c r="C28" t="s">
-        <v>18</v>
+        <v>736</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>695</v>
+        <v>453</v>
       </c>
       <c r="B29" t="s">
-        <v>684</v>
+        <v>276</v>
       </c>
       <c r="C29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>456</v>
+        <v>695</v>
       </c>
       <c r="B30" t="s">
-        <v>277</v>
+        <v>684</v>
       </c>
       <c r="C30" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="B31" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="C31" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>688</v>
+        <v>461</v>
       </c>
       <c r="B32" t="s">
-        <v>678</v>
+        <v>282</v>
       </c>
       <c r="C32" t="s">
-        <v>678</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>460</v>
+        <v>688</v>
       </c>
       <c r="B33" t="s">
-        <v>281</v>
+        <v>678</v>
       </c>
       <c r="C33" t="s">
-        <v>25</v>
+        <v>678</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B34" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C34" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>697</v>
+        <v>462</v>
       </c>
       <c r="B35" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C35" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>467</v>
+        <v>697</v>
       </c>
       <c r="B36" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C36" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B37" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B38" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C38" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -3104,7 +3110,7 @@
         <v>469</v>
       </c>
       <c r="B39" t="s">
-        <v>469</v>
+        <v>289</v>
       </c>
       <c r="C39" t="s">
         <v>33</v>
@@ -3112,156 +3118,156 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B40" t="s">
-        <v>290</v>
+        <v>469</v>
       </c>
       <c r="C40" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="B41" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C41" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B42" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C42" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>738</v>
+        <v>471</v>
       </c>
       <c r="B43" t="s">
-        <v>737</v>
+        <v>291</v>
       </c>
       <c r="C43" t="s">
-        <v>739</v>
+        <v>35</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>473</v>
+        <v>738</v>
       </c>
       <c r="B44" t="s">
-        <v>293</v>
+        <v>737</v>
       </c>
       <c r="C44" t="s">
-        <v>37</v>
+        <v>739</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B45" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>741</v>
+        <v>474</v>
       </c>
       <c r="B46" t="s">
-        <v>742</v>
+        <v>294</v>
       </c>
       <c r="C46" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>463</v>
+        <v>741</v>
       </c>
       <c r="B47" t="s">
-        <v>285</v>
+        <v>742</v>
       </c>
       <c r="C47" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="B48" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C48" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B49" t="s">
-        <v>464</v>
+        <v>286</v>
       </c>
       <c r="C49" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>693</v>
+        <v>465</v>
       </c>
       <c r="B50" t="s">
-        <v>682</v>
+        <v>464</v>
       </c>
       <c r="C50" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="B51" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="C51" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>475</v>
+        <v>691</v>
       </c>
       <c r="B52" t="s">
-        <v>295</v>
+        <v>685</v>
       </c>
       <c r="C52" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B53" t="s">
-        <v>265</v>
+        <v>295</v>
       </c>
       <c r="C53" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -3269,7 +3275,7 @@
         <v>476</v>
       </c>
       <c r="B54" t="s">
-        <v>476</v>
+        <v>265</v>
       </c>
       <c r="C54" t="s">
         <v>40</v>
@@ -3277,24 +3283,24 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B55" t="s">
-        <v>266</v>
+        <v>476</v>
       </c>
       <c r="C55" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B56" t="s">
-        <v>296</v>
+        <v>266</v>
       </c>
       <c r="C56" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -3302,7 +3308,7 @@
         <v>478</v>
       </c>
       <c r="B57" t="s">
-        <v>478</v>
+        <v>296</v>
       </c>
       <c r="C57" t="s">
         <v>42</v>
@@ -3310,79 +3316,79 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B58" t="s">
-        <v>297</v>
+        <v>478</v>
       </c>
       <c r="C58" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B59" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C59" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B60" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C60" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B61" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C61" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B62" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C62" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B63" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C63" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B64" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C64" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -3390,7 +3396,7 @@
         <v>486</v>
       </c>
       <c r="B65" t="s">
-        <v>486</v>
+        <v>304</v>
       </c>
       <c r="C65" t="s">
         <v>50</v>
@@ -3398,65 +3404,65 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B66" t="s">
-        <v>305</v>
+        <v>486</v>
       </c>
       <c r="C66" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>692</v>
+        <v>487</v>
       </c>
       <c r="B67" t="s">
-        <v>686</v>
+        <v>305</v>
       </c>
       <c r="C67" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>744</v>
+        <v>692</v>
       </c>
       <c r="B68" t="s">
-        <v>743</v>
+        <v>686</v>
       </c>
       <c r="C68" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>485</v>
+        <v>744</v>
       </c>
       <c r="B69" t="s">
-        <v>303</v>
+        <v>743</v>
       </c>
       <c r="C69" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="B70" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="C70" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>690</v>
+        <v>488</v>
       </c>
       <c r="B71" t="s">
-        <v>680</v>
+        <v>306</v>
       </c>
       <c r="C71" t="s">
         <v>53</v>
@@ -3464,277 +3470,277 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>489</v>
+        <v>690</v>
       </c>
       <c r="B72" t="s">
-        <v>307</v>
+        <v>680</v>
       </c>
       <c r="C72" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B73" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C73" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B74" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C74" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B75" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C75" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B76" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C76" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B77" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C77" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B78" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C78" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="B79" t="s">
-        <v>62</v>
+        <v>313</v>
       </c>
       <c r="C79" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B80" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C80" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
       <c r="B81" t="s">
-        <v>320</v>
+        <v>63</v>
       </c>
       <c r="C81" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B82" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C82" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B83" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C83" t="s">
-        <v>740</v>
+        <v>73</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B84" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C84" t="s">
-        <v>74</v>
+        <v>740</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B85" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C85" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B86" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C86" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="B87" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="C87" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B88" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C88" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
       <c r="B89" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C89" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>718</v>
+        <v>499</v>
       </c>
       <c r="B90" t="s">
-        <v>705</v>
+        <v>314</v>
       </c>
       <c r="C90" t="s">
-        <v>731</v>
+        <v>64</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>500</v>
+        <v>718</v>
       </c>
       <c r="B91" t="s">
-        <v>65</v>
+        <v>705</v>
       </c>
       <c r="C91" t="s">
-        <v>65</v>
+        <v>731</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B92" t="s">
-        <v>315</v>
+        <v>65</v>
       </c>
       <c r="C92" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B93" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C93" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B94" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C94" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="B95" t="s">
-        <v>69</v>
+        <v>316</v>
       </c>
       <c r="C95" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
       <c r="B96" t="s">
-        <v>494</v>
+        <v>69</v>
       </c>
       <c r="C96" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
@@ -3742,7 +3748,7 @@
         <v>494</v>
       </c>
       <c r="B97" t="s">
-        <v>681</v>
+        <v>494</v>
       </c>
       <c r="C97" t="s">
         <v>59</v>
@@ -3750,420 +3756,420 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>513</v>
+        <v>494</v>
       </c>
       <c r="B98" t="s">
-        <v>77</v>
+        <v>681</v>
       </c>
       <c r="C98" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B99" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C99" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B100" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C100" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B101" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C101" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B102" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C102" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>451</v>
+        <v>517</v>
       </c>
       <c r="B103" t="s">
-        <v>267</v>
+        <v>81</v>
       </c>
       <c r="C103" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>745</v>
+        <v>451</v>
       </c>
       <c r="B104" t="s">
-        <v>707</v>
+        <v>267</v>
       </c>
       <c r="C104" t="s">
-        <v>707</v>
+        <v>82</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>518</v>
+        <v>745</v>
       </c>
       <c r="B105" t="s">
-        <v>326</v>
+        <v>707</v>
       </c>
       <c r="C105" t="s">
-        <v>83</v>
+        <v>707</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B106" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C106" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B107" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C107" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B108" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C108" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B109" t="s">
-        <v>268</v>
+        <v>329</v>
       </c>
       <c r="C109" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B110" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C110" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B111" t="s">
-        <v>330</v>
+        <v>269</v>
       </c>
       <c r="C111" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B112" t="s">
-        <v>270</v>
+        <v>330</v>
       </c>
       <c r="C112" t="s">
-        <v>332</v>
+        <v>89</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B113" t="s">
-        <v>331</v>
+        <v>270</v>
       </c>
       <c r="C113" t="s">
-        <v>90</v>
+        <v>332</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B114" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C114" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="B115" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C115" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B116" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C116" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="B117" t="s">
-        <v>271</v>
+        <v>334</v>
       </c>
       <c r="C117" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>715</v>
+        <v>530</v>
       </c>
       <c r="B118" t="s">
-        <v>702</v>
+        <v>271</v>
       </c>
       <c r="C118" t="s">
-        <v>729</v>
+        <v>94</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>533</v>
+        <v>715</v>
       </c>
       <c r="B119" t="s">
-        <v>337</v>
+        <v>702</v>
       </c>
       <c r="C119" t="s">
-        <v>97</v>
+        <v>729</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B120" t="s">
-        <v>272</v>
+        <v>337</v>
       </c>
       <c r="C120" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B121" t="s">
-        <v>336</v>
+        <v>272</v>
       </c>
       <c r="C121" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="B122" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C122" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B123" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C123" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>719</v>
+        <v>534</v>
       </c>
       <c r="B124" t="s">
-        <v>706</v>
+        <v>338</v>
       </c>
       <c r="C124" t="s">
-        <v>732</v>
+        <v>98</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>536</v>
+        <v>719</v>
       </c>
       <c r="B125" t="s">
-        <v>340</v>
+        <v>706</v>
       </c>
       <c r="C125" t="s">
-        <v>100</v>
+        <v>732</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="B126" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C126" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B127" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C127" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B128" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C128" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B129" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C129" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B130" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C130" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B131" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C131" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B132" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C132" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B133" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C133" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B134" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C134" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B135" t="s">
-        <v>548</v>
+        <v>350</v>
       </c>
       <c r="C135" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
@@ -4171,7 +4177,7 @@
         <v>547</v>
       </c>
       <c r="B136" t="s">
-        <v>687</v>
+        <v>548</v>
       </c>
       <c r="C136" t="s">
         <v>111</v>
@@ -4179,351 +4185,351 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>537</v>
+        <v>547</v>
       </c>
       <c r="B137" t="s">
-        <v>341</v>
+        <v>687</v>
       </c>
       <c r="C137" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>549</v>
+        <v>537</v>
       </c>
       <c r="B138" t="s">
-        <v>273</v>
+        <v>341</v>
       </c>
       <c r="C138" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B139" t="s">
-        <v>351</v>
+        <v>273</v>
       </c>
       <c r="C139" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B140" t="s">
-        <v>115</v>
+        <v>351</v>
       </c>
       <c r="C140" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B141" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C141" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="B142" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C142" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B143" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C143" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B144" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C144" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B145" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C145" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B146" t="s">
-        <v>352</v>
+        <v>119</v>
       </c>
       <c r="C146" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B147" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C147" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B148" t="s">
-        <v>122</v>
+        <v>353</v>
       </c>
       <c r="C148" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>567</v>
+        <v>559</v>
       </c>
       <c r="B149" t="s">
-        <v>357</v>
+        <v>122</v>
       </c>
       <c r="C149" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B150" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C150" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="B151" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C151" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B152" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C152" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B153" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C153" t="s">
-        <v>746</v>
+        <v>135</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B154" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C154" t="s">
-        <v>136</v>
+        <v>746</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B155" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C155" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B156" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C156" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>560</v>
+        <v>576</v>
       </c>
       <c r="B157" t="s">
-        <v>354</v>
+        <v>365</v>
       </c>
       <c r="C157" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B158" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C158" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B159" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="C159" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B160" t="s">
-        <v>126</v>
+        <v>361</v>
       </c>
       <c r="C160" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B161" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C161" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B162" t="s">
-        <v>356</v>
+        <v>127</v>
       </c>
       <c r="C162" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B163" t="s">
-        <v>129</v>
+        <v>356</v>
       </c>
       <c r="C163" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="B164" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C164" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B165" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C165" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>577</v>
+        <v>570</v>
       </c>
       <c r="B166" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C166" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>714</v>
+        <v>577</v>
       </c>
       <c r="B167" t="s">
-        <v>701</v>
+        <v>139</v>
       </c>
       <c r="C167" t="s">
-        <v>728</v>
+        <v>139</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="B168" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="C168" t="s">
         <v>728</v>
@@ -4531,508 +4537,508 @@
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>578</v>
+        <v>717</v>
       </c>
       <c r="B169" t="s">
-        <v>366</v>
+        <v>704</v>
       </c>
       <c r="C169" t="s">
-        <v>140</v>
+        <v>728</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B170" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C170" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B171" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C171" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B172" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C172" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B173" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C173" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>716</v>
+        <v>582</v>
       </c>
       <c r="B174" t="s">
-        <v>703</v>
+        <v>370</v>
       </c>
       <c r="C174" t="s">
-        <v>730</v>
+        <v>144</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>583</v>
+        <v>716</v>
       </c>
       <c r="B175" t="s">
-        <v>145</v>
+        <v>703</v>
       </c>
       <c r="C175" t="s">
-        <v>145</v>
+        <v>730</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B176" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C176" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>147</v>
+        <v>584</v>
       </c>
       <c r="B177" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C177" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>585</v>
+        <v>147</v>
       </c>
       <c r="B178" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C178" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B179" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C179" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B180" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C180" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="B181" t="s">
-        <v>373</v>
+        <v>150</v>
       </c>
       <c r="C181" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B182" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C182" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>598</v>
+        <v>591</v>
       </c>
       <c r="B183" t="s">
-        <v>162</v>
+        <v>374</v>
       </c>
       <c r="C183" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>588</v>
+        <v>598</v>
       </c>
       <c r="B184" t="s">
-        <v>371</v>
+        <v>162</v>
       </c>
       <c r="C184" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B185" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C185" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
       <c r="B186" t="s">
-        <v>163</v>
+        <v>372</v>
       </c>
       <c r="C186" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>613</v>
+        <v>599</v>
       </c>
       <c r="B187" t="s">
-        <v>393</v>
+        <v>163</v>
       </c>
       <c r="C187" t="s">
-        <v>176</v>
+        <v>163</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B188" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C188" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B189" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C189" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B190" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C190" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B191" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C191" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>608</v>
+        <v>617</v>
       </c>
       <c r="B192" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="C192" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B193" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C193" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B194" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C194" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B195" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C195" t="s">
-        <v>391</v>
+        <v>174</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B196" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C196" t="s">
-        <v>175</v>
+        <v>391</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>600</v>
+        <v>612</v>
       </c>
       <c r="B197" t="s">
-        <v>164</v>
+        <v>392</v>
       </c>
       <c r="C197" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B198" t="s">
-        <v>382</v>
+        <v>164</v>
       </c>
       <c r="C198" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B199" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C199" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B200" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C200" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B201" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C201" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B202" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C202" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B203" t="s">
-        <v>170</v>
+        <v>386</v>
       </c>
       <c r="C203" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B204" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C204" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>618</v>
+        <v>607</v>
       </c>
       <c r="B205" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="C205" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B206" t="s">
-        <v>399</v>
+        <v>182</v>
       </c>
       <c r="C206" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B207" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C207" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B208" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C208" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B209" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C209" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>722</v>
+        <v>622</v>
       </c>
       <c r="B210" t="s">
-        <v>710</v>
+        <v>401</v>
       </c>
       <c r="C210" t="s">
-        <v>734</v>
+        <v>186</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>623</v>
+        <v>722</v>
       </c>
       <c r="B211" t="s">
-        <v>402</v>
+        <v>710</v>
       </c>
       <c r="C211" t="s">
-        <v>187</v>
+        <v>734</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>747</v>
+        <v>623</v>
       </c>
       <c r="B212" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C212" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>624</v>
+        <v>747</v>
       </c>
       <c r="B213" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C213" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B214" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C214" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
@@ -5040,7 +5046,7 @@
         <v>625</v>
       </c>
       <c r="B215" t="s">
-        <v>625</v>
+        <v>405</v>
       </c>
       <c r="C215" t="s">
         <v>190</v>
@@ -5048,365 +5054,365 @@
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B216" t="s">
-        <v>406</v>
+        <v>625</v>
       </c>
       <c r="C216" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B217" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C217" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B218" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C218" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B219" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C219" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>694</v>
+        <v>629</v>
       </c>
       <c r="B220" t="s">
-        <v>683</v>
+        <v>409</v>
       </c>
       <c r="C220" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>630</v>
+        <v>694</v>
       </c>
       <c r="B221" t="s">
-        <v>410</v>
+        <v>683</v>
       </c>
       <c r="C221" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B222" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C222" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B223" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C223" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>748</v>
+        <v>632</v>
       </c>
       <c r="B224" t="s">
-        <v>750</v>
+        <v>412</v>
       </c>
       <c r="C224" t="s">
-        <v>752</v>
+        <v>197</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B225" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="C225" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>633</v>
+        <v>749</v>
       </c>
       <c r="B226" t="s">
-        <v>198</v>
+        <v>751</v>
       </c>
       <c r="C226" t="s">
-        <v>198</v>
+        <v>753</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B227" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C227" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>592</v>
+        <v>634</v>
       </c>
       <c r="B228" t="s">
-        <v>375</v>
+        <v>199</v>
       </c>
       <c r="C228" t="s">
-        <v>155</v>
+        <v>199</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B229" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C229" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B230" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C230" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B231" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C231" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B232" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C232" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B233" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C233" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>754</v>
+        <v>597</v>
       </c>
       <c r="B234" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C234" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>724</v>
+        <v>754</v>
       </c>
       <c r="B235" t="s">
-        <v>713</v>
+        <v>381</v>
       </c>
       <c r="C235" t="s">
-        <v>713</v>
+        <v>161</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>635</v>
+        <v>724</v>
       </c>
       <c r="B236" t="s">
-        <v>413</v>
+        <v>713</v>
       </c>
       <c r="C236" t="s">
-        <v>200</v>
+        <v>713</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B237" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C237" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B238" t="s">
-        <v>202</v>
+        <v>414</v>
       </c>
       <c r="C238" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>641</v>
+        <v>637</v>
       </c>
       <c r="B239" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C239" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="B240" t="s">
-        <v>415</v>
+        <v>206</v>
       </c>
       <c r="C240" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B241" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C241" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>415</v>
+        <v>640</v>
       </c>
       <c r="B242" t="s">
-        <v>712</v>
+        <v>416</v>
       </c>
       <c r="C242" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>642</v>
+        <v>415</v>
       </c>
       <c r="B243" t="s">
-        <v>417</v>
+        <v>712</v>
       </c>
       <c r="C243" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="B244" t="s">
-        <v>203</v>
+        <v>417</v>
       </c>
       <c r="C244" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
       <c r="B245" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C245" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B246" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C246" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B247" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C247" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>212</v>
+        <v>646</v>
       </c>
       <c r="B248" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C248" t="s">
-        <v>696</v>
+        <v>211</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
@@ -5414,7 +5420,7 @@
         <v>212</v>
       </c>
       <c r="B249" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C249" t="s">
         <v>696</v>
@@ -5422,65 +5428,65 @@
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>647</v>
+        <v>212</v>
       </c>
       <c r="B250" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C250" t="s">
-        <v>214</v>
+        <v>696</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B251" t="s">
-        <v>419</v>
+        <v>214</v>
       </c>
       <c r="C251" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B252" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C252" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B253" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C253" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="B254" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="C254" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
+        <v>645</v>
+      </c>
+      <c r="B255" t="s">
         <v>418</v>
-      </c>
-      <c r="B255" t="s">
-        <v>698</v>
       </c>
       <c r="C255" t="s">
         <v>210</v>
@@ -5488,348 +5494,359 @@
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>218</v>
+        <v>418</v>
       </c>
       <c r="B256" t="s">
-        <v>218</v>
+        <v>698</v>
       </c>
       <c r="C256" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>720</v>
+        <v>218</v>
       </c>
       <c r="B257" t="s">
-        <v>708</v>
+        <v>218</v>
       </c>
       <c r="C257" t="s">
-        <v>708</v>
+        <v>218</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>652</v>
+        <v>720</v>
       </c>
       <c r="B258" t="s">
-        <v>220</v>
+        <v>708</v>
       </c>
       <c r="C258" t="s">
-        <v>220</v>
+        <v>708</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B259" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C259" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="B260" t="s">
-        <v>422</v>
+        <v>221</v>
       </c>
       <c r="C260" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
       <c r="B261" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="C261" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="B262" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="C262" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="B263" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C263" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="B264" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="C264" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B265" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C265" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="B266" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="C266" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="B267" t="s">
-        <v>423</v>
+        <v>434</v>
       </c>
       <c r="C267" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>721</v>
+        <v>655</v>
       </c>
       <c r="B268" t="s">
-        <v>709</v>
+        <v>423</v>
       </c>
       <c r="C268" t="s">
-        <v>733</v>
+        <v>222</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>657</v>
+        <v>721</v>
       </c>
       <c r="B269" t="s">
-        <v>425</v>
+        <v>709</v>
       </c>
       <c r="C269" t="s">
-        <v>223</v>
+        <v>733</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="B270" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C270" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B271" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C271" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="B272" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="C272" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>723</v>
+        <v>663</v>
       </c>
       <c r="B273" t="s">
-        <v>711</v>
+        <v>432</v>
       </c>
       <c r="C273" t="s">
-        <v>735</v>
+        <v>229</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="B274" t="s">
-        <v>699</v>
+        <v>711</v>
       </c>
       <c r="C274" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>664</v>
+        <v>726</v>
       </c>
       <c r="B275" t="s">
-        <v>433</v>
+        <v>699</v>
       </c>
       <c r="C275" t="s">
-        <v>230</v>
+        <v>727</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B276" t="s">
-        <v>232</v>
+        <v>433</v>
       </c>
       <c r="C276" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B277" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C277" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B278" t="s">
-        <v>435</v>
+        <v>233</v>
       </c>
       <c r="C278" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B279" t="s">
-        <v>670</v>
+        <v>435</v>
       </c>
       <c r="C279" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B280" t="s">
-        <v>436</v>
+        <v>670</v>
       </c>
       <c r="C280" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B281" t="s">
-        <v>237</v>
+        <v>436</v>
       </c>
       <c r="C281" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B282" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C282" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="B283" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C283" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B284" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C284" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B285" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C285" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
+        <v>676</v>
+      </c>
+      <c r="B286" t="s">
+        <v>241</v>
+      </c>
+      <c r="C286" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
         <v>677</v>
       </c>
-      <c r="B286" t="s">
+      <c r="B287" t="s">
         <v>242</v>
       </c>
-      <c r="C286" t="s">
+      <c r="C287" t="s">
         <v>242</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C286">
-    <sortCondition ref="A2:A286"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C287">
+    <sortCondition ref="A2:A287"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Walka z św.. świętych, świętego i świętej
</commit_message>
<xml_diff>
--- a/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
+++ b/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\AddressLibrary\AddressLibrary\AppData\Dictionaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC0592E-21D0-4D0A-B426-C1DD3D07F832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F1A3CE-7DEB-4A13-BDDB-F507A8595FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="759">
   <si>
     <t>abp</t>
   </si>
@@ -2307,6 +2307,12 @@
   </si>
   <si>
     <t>biskupów</t>
+  </si>
+  <si>
+    <t>prezydentów Rzeczpospolitej Polskiej</t>
+  </si>
+  <si>
+    <t>prezydenci Rzeczpospolitej Polskiej</t>
   </si>
 </sst>
 </file>
@@ -2679,7 +2685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD74A5C-AF8A-492F-8246-0B7893A73121}">
-  <dimension ref="A1:C287"/>
+  <dimension ref="A1:C288"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" customWidth="1"/>
@@ -3833,343 +3839,343 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>745</v>
+        <v>518</v>
       </c>
       <c r="B105" t="s">
-        <v>707</v>
+        <v>326</v>
       </c>
       <c r="C105" t="s">
-        <v>707</v>
+        <v>83</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B106" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C106" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B107" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C107" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B108" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C108" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B109" t="s">
-        <v>329</v>
+        <v>268</v>
       </c>
       <c r="C109" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B110" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C110" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B111" t="s">
-        <v>269</v>
+        <v>330</v>
       </c>
       <c r="C111" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B112" t="s">
-        <v>330</v>
+        <v>270</v>
       </c>
       <c r="C112" t="s">
-        <v>89</v>
+        <v>332</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B113" t="s">
-        <v>270</v>
+        <v>331</v>
       </c>
       <c r="C113" t="s">
-        <v>332</v>
+        <v>90</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B114" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C114" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B115" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C115" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B116" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C116" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B117" t="s">
-        <v>334</v>
+        <v>271</v>
       </c>
       <c r="C117" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>530</v>
+        <v>715</v>
       </c>
       <c r="B118" t="s">
-        <v>271</v>
+        <v>702</v>
       </c>
       <c r="C118" t="s">
-        <v>94</v>
+        <v>729</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>715</v>
+        <v>533</v>
       </c>
       <c r="B119" t="s">
-        <v>702</v>
+        <v>337</v>
       </c>
       <c r="C119" t="s">
-        <v>729</v>
+        <v>97</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="B120" t="s">
-        <v>337</v>
+        <v>272</v>
       </c>
       <c r="C120" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B121" t="s">
-        <v>272</v>
+        <v>336</v>
       </c>
       <c r="C121" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B122" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="C122" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B123" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C123" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>534</v>
+        <v>719</v>
       </c>
       <c r="B124" t="s">
-        <v>338</v>
+        <v>706</v>
       </c>
       <c r="C124" t="s">
-        <v>98</v>
+        <v>732</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>719</v>
+        <v>536</v>
       </c>
       <c r="B125" t="s">
-        <v>706</v>
+        <v>340</v>
       </c>
       <c r="C125" t="s">
-        <v>732</v>
+        <v>100</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B126" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C126" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B127" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C127" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B128" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C128" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B129" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C129" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B130" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C130" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B131" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C131" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B132" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C132" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B133" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C133" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B134" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C134" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B135" t="s">
-        <v>350</v>
+        <v>548</v>
       </c>
       <c r="C135" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
@@ -4177,7 +4183,7 @@
         <v>547</v>
       </c>
       <c r="B136" t="s">
-        <v>548</v>
+        <v>687</v>
       </c>
       <c r="C136" t="s">
         <v>111</v>
@@ -4185,68 +4191,68 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>547</v>
+        <v>537</v>
       </c>
       <c r="B137" t="s">
-        <v>687</v>
+        <v>341</v>
       </c>
       <c r="C137" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>537</v>
+        <v>549</v>
       </c>
       <c r="B138" t="s">
-        <v>341</v>
+        <v>273</v>
       </c>
       <c r="C138" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B139" t="s">
-        <v>273</v>
+        <v>351</v>
       </c>
       <c r="C139" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B140" t="s">
-        <v>351</v>
+        <v>115</v>
       </c>
       <c r="C140" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B141" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C141" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>551</v>
+        <v>745</v>
       </c>
       <c r="B142" t="s">
-        <v>114</v>
+        <v>707</v>
       </c>
       <c r="C142" t="s">
-        <v>114</v>
+        <v>707</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
@@ -4977,79 +4983,79 @@
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>621</v>
+        <v>758</v>
       </c>
       <c r="B209" t="s">
-        <v>400</v>
+        <v>757</v>
       </c>
       <c r="C209" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B210" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C210" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>722</v>
+        <v>622</v>
       </c>
       <c r="B211" t="s">
-        <v>710</v>
+        <v>401</v>
       </c>
       <c r="C211" t="s">
-        <v>734</v>
+        <v>186</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>623</v>
+        <v>722</v>
       </c>
       <c r="B212" t="s">
-        <v>402</v>
+        <v>710</v>
       </c>
       <c r="C212" t="s">
-        <v>187</v>
+        <v>734</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>747</v>
+        <v>623</v>
       </c>
       <c r="B213" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C213" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>624</v>
+        <v>747</v>
       </c>
       <c r="B214" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C214" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B215" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C215" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
@@ -5057,7 +5063,7 @@
         <v>625</v>
       </c>
       <c r="B216" t="s">
-        <v>625</v>
+        <v>405</v>
       </c>
       <c r="C216" t="s">
         <v>190</v>
@@ -5065,365 +5071,365 @@
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B217" t="s">
-        <v>406</v>
+        <v>625</v>
       </c>
       <c r="C217" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B218" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C218" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B219" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C219" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B220" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C220" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>694</v>
+        <v>629</v>
       </c>
       <c r="B221" t="s">
-        <v>683</v>
+        <v>409</v>
       </c>
       <c r="C221" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>630</v>
+        <v>694</v>
       </c>
       <c r="B222" t="s">
-        <v>410</v>
+        <v>683</v>
       </c>
       <c r="C222" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B223" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C223" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>632</v>
+        <v>748</v>
       </c>
       <c r="B224" t="s">
-        <v>412</v>
+        <v>750</v>
       </c>
       <c r="C224" t="s">
-        <v>197</v>
+        <v>752</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B225" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C225" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>749</v>
+        <v>631</v>
       </c>
       <c r="B226" t="s">
-        <v>751</v>
+        <v>411</v>
       </c>
       <c r="C226" t="s">
-        <v>753</v>
+        <v>196</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B227" t="s">
-        <v>198</v>
+        <v>412</v>
       </c>
       <c r="C227" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B228" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C228" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>592</v>
+        <v>634</v>
       </c>
       <c r="B229" t="s">
-        <v>375</v>
+        <v>199</v>
       </c>
       <c r="C229" t="s">
-        <v>155</v>
+        <v>199</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B230" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C230" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B231" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C231" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B232" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C232" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B233" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C233" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B234" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C234" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>754</v>
+        <v>597</v>
       </c>
       <c r="B235" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C235" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>724</v>
+        <v>754</v>
       </c>
       <c r="B236" t="s">
-        <v>713</v>
+        <v>381</v>
       </c>
       <c r="C236" t="s">
-        <v>713</v>
+        <v>161</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>635</v>
+        <v>724</v>
       </c>
       <c r="B237" t="s">
-        <v>413</v>
+        <v>713</v>
       </c>
       <c r="C237" t="s">
-        <v>200</v>
+        <v>713</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B238" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C238" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B239" t="s">
-        <v>202</v>
+        <v>414</v>
       </c>
       <c r="C239" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>641</v>
+        <v>637</v>
       </c>
       <c r="B240" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C240" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="B241" t="s">
-        <v>415</v>
+        <v>206</v>
       </c>
       <c r="C241" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B242" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C242" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>415</v>
+        <v>640</v>
       </c>
       <c r="B243" t="s">
-        <v>712</v>
+        <v>416</v>
       </c>
       <c r="C243" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>642</v>
+        <v>415</v>
       </c>
       <c r="B244" t="s">
-        <v>417</v>
+        <v>712</v>
       </c>
       <c r="C244" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="B245" t="s">
-        <v>203</v>
+        <v>417</v>
       </c>
       <c r="C245" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
       <c r="B246" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C246" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B247" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C247" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B248" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C248" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>212</v>
+        <v>646</v>
       </c>
       <c r="B249" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C249" t="s">
-        <v>696</v>
+        <v>211</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
@@ -5431,7 +5437,7 @@
         <v>212</v>
       </c>
       <c r="B250" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C250" t="s">
         <v>696</v>
@@ -5439,65 +5445,65 @@
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>647</v>
+        <v>212</v>
       </c>
       <c r="B251" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C251" t="s">
-        <v>214</v>
+        <v>696</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B252" t="s">
-        <v>419</v>
+        <v>214</v>
       </c>
       <c r="C252" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B253" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C253" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B254" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C254" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="B255" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="C255" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
+        <v>645</v>
+      </c>
+      <c r="B256" t="s">
         <v>418</v>
-      </c>
-      <c r="B256" t="s">
-        <v>698</v>
       </c>
       <c r="C256" t="s">
         <v>210</v>
@@ -5505,348 +5511,359 @@
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>218</v>
+        <v>418</v>
       </c>
       <c r="B257" t="s">
-        <v>218</v>
+        <v>698</v>
       </c>
       <c r="C257" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>720</v>
+        <v>218</v>
       </c>
       <c r="B258" t="s">
-        <v>708</v>
+        <v>218</v>
       </c>
       <c r="C258" t="s">
-        <v>708</v>
+        <v>218</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>652</v>
+        <v>720</v>
       </c>
       <c r="B259" t="s">
-        <v>220</v>
+        <v>708</v>
       </c>
       <c r="C259" t="s">
-        <v>220</v>
+        <v>708</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B260" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C260" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="B261" t="s">
-        <v>422</v>
+        <v>221</v>
       </c>
       <c r="C261" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
       <c r="B262" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="C262" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="B263" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="C263" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="B264" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C264" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>661</v>
+        <v>654</v>
       </c>
       <c r="B265" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="C265" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B266" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C266" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="B267" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="C267" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
       <c r="B268" t="s">
-        <v>423</v>
+        <v>434</v>
       </c>
       <c r="C268" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>721</v>
+        <v>655</v>
       </c>
       <c r="B269" t="s">
-        <v>709</v>
+        <v>423</v>
       </c>
       <c r="C269" t="s">
-        <v>733</v>
+        <v>222</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>657</v>
+        <v>721</v>
       </c>
       <c r="B270" t="s">
-        <v>425</v>
+        <v>709</v>
       </c>
       <c r="C270" t="s">
-        <v>223</v>
+        <v>733</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="B271" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C271" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B272" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C272" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="B273" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="C273" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>723</v>
+        <v>663</v>
       </c>
       <c r="B274" t="s">
-        <v>711</v>
+        <v>432</v>
       </c>
       <c r="C274" t="s">
-        <v>735</v>
+        <v>229</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="B275" t="s">
-        <v>699</v>
+        <v>711</v>
       </c>
       <c r="C275" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>664</v>
+        <v>726</v>
       </c>
       <c r="B276" t="s">
-        <v>433</v>
+        <v>699</v>
       </c>
       <c r="C276" t="s">
-        <v>230</v>
+        <v>727</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B277" t="s">
-        <v>232</v>
+        <v>433</v>
       </c>
       <c r="C277" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B278" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C278" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B279" t="s">
-        <v>435</v>
+        <v>233</v>
       </c>
       <c r="C279" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B280" t="s">
-        <v>670</v>
+        <v>435</v>
       </c>
       <c r="C280" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B281" t="s">
-        <v>436</v>
+        <v>670</v>
       </c>
       <c r="C281" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B282" t="s">
-        <v>237</v>
+        <v>436</v>
       </c>
       <c r="C282" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B283" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C283" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="B284" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C284" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B285" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C285" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B286" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C286" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
+        <v>676</v>
+      </c>
+      <c r="B287" t="s">
+        <v>241</v>
+      </c>
+      <c r="C287" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
         <v>677</v>
       </c>
-      <c r="B287" t="s">
+      <c r="B288" t="s">
         <v>242</v>
       </c>
-      <c r="C287" t="s">
+      <c r="C288" t="s">
         <v>242</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C287">
-    <sortCondition ref="A2:A287"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C288">
+    <sortCondition ref="A2:A288"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Przed zmianą łączenia ładowania załączników i hierarchii
</commit_message>
<xml_diff>
--- a/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
+++ b/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\AddressLibrary\AddressLibrary\AppData\Dictionaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F1A3CE-7DEB-4A13-BDDB-F507A8595FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB331D2-911B-4F7B-AE19-50C0C303EAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="759">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="761">
   <si>
     <t>abp</t>
   </si>
@@ -650,12 +650,6 @@
     <t>rodu</t>
   </si>
   <si>
-    <t>rodz.</t>
-  </si>
-  <si>
-    <t>rodz. hr.</t>
-  </si>
-  <si>
     <t>rodzeństwa</t>
   </si>
   <si>
@@ -2313,6 +2307,18 @@
   </si>
   <si>
     <t>prezydenci Rzeczpospolitej Polskiej</t>
+  </si>
+  <si>
+    <t>rodziny hr.</t>
+  </si>
+  <si>
+    <t>święta rodzina</t>
+  </si>
+  <si>
+    <t>świętej rodziny</t>
+  </si>
+  <si>
+    <t>św. rodziny</t>
   </si>
 </sst>
 </file>
@@ -2685,7 +2691,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD74A5C-AF8A-492F-8246-0B7893A73121}">
-  <dimension ref="A1:C288"/>
+  <dimension ref="A1:C289"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" customWidth="1"/>
@@ -2695,21 +2701,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
@@ -2717,10 +2723,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="B3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -2728,10 +2734,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B4" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -2739,10 +2745,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B5" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -2750,10 +2756,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="B6" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
@@ -2761,10 +2767,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B7" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C7" t="s">
         <v>0</v>
@@ -2772,10 +2778,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -2783,10 +2789,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B9" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C9" t="s">
         <v>2</v>
@@ -2794,10 +2800,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B10" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
@@ -2805,7 +2811,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B11" t="s">
         <v>8</v>
@@ -2816,7 +2822,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B12" t="s">
         <v>9</v>
@@ -2827,10 +2833,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="B13" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C13" t="s">
         <v>24</v>
@@ -2838,10 +2844,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="B14" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="C14" t="s">
         <v>24</v>
@@ -2849,10 +2855,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B15" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C15" t="s">
         <v>10</v>
@@ -2860,10 +2866,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B16" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C16" t="s">
         <v>10</v>
@@ -2871,10 +2877,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="B17" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C17" t="s">
         <v>14</v>
@@ -2882,10 +2888,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="B18" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C18" t="s">
         <v>20</v>
@@ -2893,10 +2899,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B19" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C19" t="s">
         <v>22</v>
@@ -2904,10 +2910,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B20" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C20" t="s">
         <v>23</v>
@@ -2915,10 +2921,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B21" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="C21" t="s">
         <v>10</v>
@@ -2926,10 +2932,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B22" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C22" t="s">
         <v>11</v>
@@ -2937,10 +2943,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B23" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C23" t="s">
         <v>12</v>
@@ -2948,10 +2954,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B24" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C24" t="s">
         <v>13</v>
@@ -2959,10 +2965,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B25" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C25" t="s">
         <v>15</v>
@@ -2970,10 +2976,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="B26" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C26" t="s">
         <v>16</v>
@@ -2981,10 +2987,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="B27" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C27" t="s">
         <v>17</v>
@@ -2992,21 +2998,21 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="B28" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="C28" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="B29" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C29" t="s">
         <v>18</v>
@@ -3014,10 +3020,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="B30" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="C30" t="s">
         <v>19</v>
@@ -3025,10 +3031,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="B31" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C31" t="s">
         <v>21</v>
@@ -3036,10 +3042,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="B32" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C32" t="s">
         <v>26</v>
@@ -3047,21 +3053,21 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B33" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="C33" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B34" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C34" t="s">
         <v>25</v>
@@ -3069,10 +3075,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B35" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C35" t="s">
         <v>27</v>
@@ -3080,10 +3086,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="B36" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C36" t="s">
         <v>28</v>
@@ -3091,10 +3097,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B37" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C37" t="s">
         <v>31</v>
@@ -3102,10 +3108,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B38" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C38" t="s">
         <v>32</v>
@@ -3113,10 +3119,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B39" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C39" t="s">
         <v>33</v>
@@ -3124,10 +3130,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B40" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="C40" t="s">
         <v>33</v>
@@ -3135,10 +3141,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="B41" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C41" t="s">
         <v>34</v>
@@ -3146,10 +3152,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="B42" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C42" t="s">
         <v>36</v>
@@ -3157,10 +3163,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B43" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C43" t="s">
         <v>35</v>
@@ -3168,21 +3174,21 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="B44" t="s">
+        <v>735</v>
+      </c>
+      <c r="C44" t="s">
         <v>737</v>
-      </c>
-      <c r="C44" t="s">
-        <v>739</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B45" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C45" t="s">
         <v>37</v>
@@ -3190,10 +3196,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B46" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C46" t="s">
         <v>38</v>
@@ -3201,10 +3207,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="B47" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="C47" t="s">
         <v>33</v>
@@ -3212,10 +3218,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="B48" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C48" t="s">
         <v>29</v>
@@ -3223,10 +3229,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B49" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C49" t="s">
         <v>30</v>
@@ -3234,10 +3240,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="B50" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="C50" t="s">
         <v>29</v>
@@ -3245,10 +3251,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="B51" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="C51" t="s">
         <v>30</v>
@@ -3256,10 +3262,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B52" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="C52" t="s">
         <v>29</v>
@@ -3267,10 +3273,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B53" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C53" t="s">
         <v>39</v>
@@ -3278,10 +3284,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B54" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C54" t="s">
         <v>40</v>
@@ -3289,10 +3295,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B55" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="C55" t="s">
         <v>40</v>
@@ -3300,10 +3306,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B56" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C56" t="s">
         <v>41</v>
@@ -3311,10 +3317,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B57" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C57" t="s">
         <v>42</v>
@@ -3322,10 +3328,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B58" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="C58" t="s">
         <v>42</v>
@@ -3333,10 +3339,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B59" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C59" t="s">
         <v>43</v>
@@ -3344,10 +3350,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B60" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C60" t="s">
         <v>44</v>
@@ -3355,10 +3361,10 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B61" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C61" t="s">
         <v>45</v>
@@ -3366,10 +3372,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="B62" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C62" t="s">
         <v>46</v>
@@ -3377,10 +3383,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B63" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C63" t="s">
         <v>47</v>
@@ -3388,10 +3394,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B64" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C64" t="s">
         <v>48</v>
@@ -3399,10 +3405,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B65" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C65" t="s">
         <v>50</v>
@@ -3410,10 +3416,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B66" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C66" t="s">
         <v>50</v>
@@ -3421,10 +3427,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B67" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C67" t="s">
         <v>51</v>
@@ -3432,10 +3438,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="B68" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="C68" t="s">
         <v>52</v>
@@ -3443,10 +3449,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="B69" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="C69" t="s">
         <v>50</v>
@@ -3454,10 +3460,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="B70" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C70" t="s">
         <v>49</v>
@@ -3465,10 +3471,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="B71" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C71" t="s">
         <v>53</v>
@@ -3476,10 +3482,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="B72" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C72" t="s">
         <v>53</v>
@@ -3487,10 +3493,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B73" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C73" t="s">
         <v>54</v>
@@ -3498,10 +3504,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="B74" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C74" t="s">
         <v>55</v>
@@ -3509,10 +3515,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B75" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C75" t="s">
         <v>56</v>
@@ -3520,10 +3526,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="B76" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C76" t="s">
         <v>57</v>
@@ -3531,10 +3537,10 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B77" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C77" t="s">
         <v>58</v>
@@ -3542,10 +3548,10 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="B78" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C78" t="s">
         <v>61</v>
@@ -3553,10 +3559,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="B79" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C79" t="s">
         <v>60</v>
@@ -3564,7 +3570,7 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="B80" t="s">
         <v>62</v>
@@ -3575,7 +3581,7 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="B81" t="s">
         <v>63</v>
@@ -3586,10 +3592,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B82" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C82" t="s">
         <v>72</v>
@@ -3597,10 +3603,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="B83" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C83" t="s">
         <v>73</v>
@@ -3608,21 +3614,21 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B84" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C84" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B85" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C85" t="s">
         <v>74</v>
@@ -3630,10 +3636,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B86" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C86" t="s">
         <v>75</v>
@@ -3641,10 +3647,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="B87" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C87" t="s">
         <v>76</v>
@@ -3652,10 +3658,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B88" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C88" t="s">
         <v>70</v>
@@ -3663,10 +3669,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="B89" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C89" t="s">
         <v>71</v>
@@ -3674,10 +3680,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="B90" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C90" t="s">
         <v>64</v>
@@ -3685,18 +3691,18 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="B91" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="C91" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="B92" t="s">
         <v>65</v>
@@ -3707,10 +3713,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B93" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C93" t="s">
         <v>66</v>
@@ -3718,10 +3724,10 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B94" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C94" t="s">
         <v>68</v>
@@ -3729,10 +3735,10 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="B95" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C95" t="s">
         <v>67</v>
@@ -3740,7 +3746,7 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="B96" t="s">
         <v>69</v>
@@ -3751,10 +3757,10 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B97" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C97" t="s">
         <v>59</v>
@@ -3762,10 +3768,10 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B98" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="C98" t="s">
         <v>59</v>
@@ -3773,7 +3779,7 @@
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="B99" t="s">
         <v>77</v>
@@ -3784,7 +3790,7 @@
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="B100" t="s">
         <v>78</v>
@@ -3795,7 +3801,7 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B101" t="s">
         <v>79</v>
@@ -3806,7 +3812,7 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="B102" t="s">
         <v>80</v>
@@ -3817,7 +3823,7 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="B103" t="s">
         <v>81</v>
@@ -3828,10 +3834,10 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B104" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C104" t="s">
         <v>82</v>
@@ -3839,10 +3845,10 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="B105" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C105" t="s">
         <v>83</v>
@@ -3850,10 +3856,10 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="B106" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C106" t="s">
         <v>84</v>
@@ -3861,10 +3867,10 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="B107" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C107" t="s">
         <v>85</v>
@@ -3872,10 +3878,10 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B108" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C108" t="s">
         <v>86</v>
@@ -3883,10 +3889,10 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="B109" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C109" t="s">
         <v>87</v>
@@ -3894,10 +3900,10 @@
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="B110" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C110" t="s">
         <v>88</v>
@@ -3905,10 +3911,10 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="B111" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C111" t="s">
         <v>89</v>
@@ -3916,21 +3922,21 @@
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="B112" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C112" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="B113" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C113" t="s">
         <v>90</v>
@@ -3938,10 +3944,10 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B114" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C114" t="s">
         <v>91</v>
@@ -3949,10 +3955,10 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="B115" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C115" t="s">
         <v>93</v>
@@ -3960,10 +3966,10 @@
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="B116" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C116" t="s">
         <v>92</v>
@@ -3971,10 +3977,10 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="B117" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C117" t="s">
         <v>94</v>
@@ -3982,21 +3988,21 @@
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="B118" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="C118" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="B119" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C119" t="s">
         <v>97</v>
@@ -4004,10 +4010,10 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="B120" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C120" t="s">
         <v>95</v>
@@ -4015,10 +4021,10 @@
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="B121" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C121" t="s">
         <v>96</v>
@@ -4026,10 +4032,10 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B122" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C122" t="s">
         <v>99</v>
@@ -4037,10 +4043,10 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B123" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C123" t="s">
         <v>98</v>
@@ -4048,21 +4054,21 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="B124" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="C124" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="B125" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C125" t="s">
         <v>100</v>
@@ -4070,10 +4076,10 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="B126" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C126" t="s">
         <v>103</v>
@@ -4081,10 +4087,10 @@
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="B127" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C127" t="s">
         <v>102</v>
@@ -4092,10 +4098,10 @@
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B128" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C128" t="s">
         <v>104</v>
@@ -4103,10 +4109,10 @@
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="B129" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C129" t="s">
         <v>105</v>
@@ -4114,10 +4120,10 @@
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B130" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C130" t="s">
         <v>106</v>
@@ -4125,10 +4131,10 @@
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B131" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C131" t="s">
         <v>107</v>
@@ -4136,10 +4142,10 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B132" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C132" t="s">
         <v>108</v>
@@ -4147,10 +4153,10 @@
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="B133" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C133" t="s">
         <v>109</v>
@@ -4158,10 +4164,10 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B134" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C134" t="s">
         <v>110</v>
@@ -4169,10 +4175,10 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="B135" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="C135" t="s">
         <v>111</v>
@@ -4180,10 +4186,10 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="B136" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="C136" t="s">
         <v>111</v>
@@ -4191,10 +4197,10 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="B137" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C137" t="s">
         <v>101</v>
@@ -4202,10 +4208,10 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="B138" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C138" t="s">
         <v>112</v>
@@ -4213,10 +4219,10 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="B139" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C139" t="s">
         <v>113</v>
@@ -4224,7 +4230,7 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B140" t="s">
         <v>115</v>
@@ -4235,7 +4241,7 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B141" t="s">
         <v>114</v>
@@ -4246,18 +4252,18 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="B142" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="C142" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="B143" t="s">
         <v>116</v>
@@ -4268,7 +4274,7 @@
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B144" t="s">
         <v>117</v>
@@ -4279,7 +4285,7 @@
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="B145" t="s">
         <v>118</v>
@@ -4290,7 +4296,7 @@
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="B146" t="s">
         <v>119</v>
@@ -4301,10 +4307,10 @@
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="B147" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C147" t="s">
         <v>120</v>
@@ -4312,10 +4318,10 @@
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B148" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C148" t="s">
         <v>121</v>
@@ -4323,7 +4329,7 @@
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="B149" t="s">
         <v>122</v>
@@ -4334,10 +4340,10 @@
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B150" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C150" t="s">
         <v>130</v>
@@ -4345,10 +4351,10 @@
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="B151" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C151" t="s">
         <v>131</v>
@@ -4356,10 +4362,10 @@
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="B152" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C152" t="s">
         <v>134</v>
@@ -4367,10 +4373,10 @@
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B153" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C153" t="s">
         <v>135</v>
@@ -4378,21 +4384,21 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="B154" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C154" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B155" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C155" t="s">
         <v>136</v>
@@ -4400,10 +4406,10 @@
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="B156" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C156" t="s">
         <v>137</v>
@@ -4411,10 +4417,10 @@
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B157" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C157" t="s">
         <v>138</v>
@@ -4422,10 +4428,10 @@
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B158" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C158" t="s">
         <v>123</v>
@@ -4433,10 +4439,10 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B159" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C159" t="s">
         <v>124</v>
@@ -4444,10 +4450,10 @@
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="B160" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C160" t="s">
         <v>125</v>
@@ -4455,7 +4461,7 @@
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B161" t="s">
         <v>126</v>
@@ -4466,7 +4472,7 @@
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="B162" t="s">
         <v>127</v>
@@ -4477,10 +4483,10 @@
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="B163" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C163" t="s">
         <v>128</v>
@@ -4488,7 +4494,7 @@
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="B164" t="s">
         <v>129</v>
@@ -4499,7 +4505,7 @@
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="B165" t="s">
         <v>132</v>
@@ -4510,7 +4516,7 @@
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="B166" t="s">
         <v>133</v>
@@ -4521,7 +4527,7 @@
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="B167" t="s">
         <v>139</v>
@@ -4532,32 +4538,32 @@
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="B168" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="C168" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="B169" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="C169" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B170" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C170" t="s">
         <v>140</v>
@@ -4565,10 +4571,10 @@
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="B171" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C171" t="s">
         <v>141</v>
@@ -4576,10 +4582,10 @@
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B172" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C172" t="s">
         <v>142</v>
@@ -4587,10 +4593,10 @@
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="B173" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C173" t="s">
         <v>143</v>
@@ -4598,10 +4604,10 @@
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B174" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C174" t="s">
         <v>144</v>
@@ -4609,18 +4615,18 @@
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="B175" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="C175" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B176" t="s">
         <v>145</v>
@@ -4631,7 +4637,7 @@
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B177" t="s">
         <v>146</v>
@@ -4653,7 +4659,7 @@
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B179" t="s">
         <v>148</v>
@@ -4664,7 +4670,7 @@
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B180" t="s">
         <v>149</v>
@@ -4675,7 +4681,7 @@
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="B181" t="s">
         <v>150</v>
@@ -4686,10 +4692,10 @@
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B182" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C182" t="s">
         <v>153</v>
@@ -4697,10 +4703,10 @@
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B183" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C183" t="s">
         <v>154</v>
@@ -4708,7 +4714,7 @@
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="B184" t="s">
         <v>162</v>
@@ -4719,10 +4725,10 @@
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B185" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C185" t="s">
         <v>151</v>
@@ -4730,10 +4736,10 @@
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="B186" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C186" t="s">
         <v>152</v>
@@ -4741,7 +4747,7 @@
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="B187" t="s">
         <v>163</v>
@@ -4752,10 +4758,10 @@
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="B188" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C188" t="s">
         <v>176</v>
@@ -4763,10 +4769,10 @@
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="B189" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C189" t="s">
         <v>177</v>
@@ -4774,10 +4780,10 @@
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B190" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C190" t="s">
         <v>178</v>
@@ -4785,10 +4791,10 @@
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="B191" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C191" t="s">
         <v>179</v>
@@ -4796,10 +4802,10 @@
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="B192" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C192" t="s">
         <v>180</v>
@@ -4807,10 +4813,10 @@
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B193" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C193" t="s">
         <v>172</v>
@@ -4818,10 +4824,10 @@
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="B194" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C194" t="s">
         <v>173</v>
@@ -4829,10 +4835,10 @@
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="B195" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C195" t="s">
         <v>174</v>
@@ -4840,21 +4846,21 @@
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="B196" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C196" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="B197" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C197" t="s">
         <v>175</v>
@@ -4862,7 +4868,7 @@
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="B198" t="s">
         <v>164</v>
@@ -4873,10 +4879,10 @@
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B199" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C199" t="s">
         <v>165</v>
@@ -4884,10 +4890,10 @@
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="B200" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="C200" t="s">
         <v>166</v>
@@ -4895,10 +4901,10 @@
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B201" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C201" t="s">
         <v>167</v>
@@ -4906,10 +4912,10 @@
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B202" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C202" t="s">
         <v>168</v>
@@ -4917,10 +4923,10 @@
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B203" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C203" t="s">
         <v>169</v>
@@ -4928,7 +4934,7 @@
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B204" t="s">
         <v>170</v>
@@ -4939,7 +4945,7 @@
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B205" t="s">
         <v>171</v>
@@ -4950,7 +4956,7 @@
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="B206" t="s">
         <v>182</v>
@@ -4961,10 +4967,10 @@
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B207" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C207" t="s">
         <v>183</v>
@@ -4972,10 +4978,10 @@
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="B208" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="C208" t="s">
         <v>184</v>
@@ -4983,10 +4989,10 @@
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="B209" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="C209" t="s">
         <v>187</v>
@@ -4994,10 +5000,10 @@
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="B210" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C210" t="s">
         <v>185</v>
@@ -5005,10 +5011,10 @@
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B211" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C211" t="s">
         <v>186</v>
@@ -5016,21 +5022,21 @@
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B212" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="C212" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="B213" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C213" t="s">
         <v>187</v>
@@ -5038,10 +5044,10 @@
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="B214" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C214" t="s">
         <v>188</v>
@@ -5049,10 +5055,10 @@
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="B215" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C215" t="s">
         <v>189</v>
@@ -5060,10 +5066,10 @@
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B216" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C216" t="s">
         <v>190</v>
@@ -5071,10 +5077,10 @@
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B217" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C217" t="s">
         <v>190</v>
@@ -5082,10 +5088,10 @@
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="B218" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C218" t="s">
         <v>191</v>
@@ -5093,10 +5099,10 @@
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="B219" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C219" t="s">
         <v>192</v>
@@ -5104,10 +5110,10 @@
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B220" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C220" t="s">
         <v>193</v>
@@ -5115,10 +5121,10 @@
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="B221" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C221" t="s">
         <v>194</v>
@@ -5126,10 +5132,10 @@
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="B222" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="C222" t="s">
         <v>190</v>
@@ -5137,10 +5143,10 @@
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B223" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C223" t="s">
         <v>195</v>
@@ -5148,32 +5154,32 @@
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
+        <v>746</v>
+      </c>
+      <c r="B224" t="s">
         <v>748</v>
       </c>
-      <c r="B224" t="s">
+      <c r="C224" t="s">
         <v>750</v>
-      </c>
-      <c r="C224" t="s">
-        <v>752</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
+        <v>747</v>
+      </c>
+      <c r="B225" t="s">
         <v>749</v>
       </c>
-      <c r="B225" t="s">
+      <c r="C225" t="s">
         <v>751</v>
-      </c>
-      <c r="C225" t="s">
-        <v>753</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="B226" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C226" t="s">
         <v>196</v>
@@ -5181,10 +5187,10 @@
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B227" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="C227" t="s">
         <v>197</v>
@@ -5192,7 +5198,7 @@
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="B228" t="s">
         <v>198</v>
@@ -5203,7 +5209,7 @@
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="B229" t="s">
         <v>199</v>
@@ -5214,10 +5220,10 @@
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="B230" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C230" t="s">
         <v>155</v>
@@ -5225,10 +5231,10 @@
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B231" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C231" t="s">
         <v>156</v>
@@ -5236,10 +5242,10 @@
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="B232" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C232" t="s">
         <v>157</v>
@@ -5247,10 +5253,10 @@
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B233" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C233" t="s">
         <v>158</v>
@@ -5258,10 +5264,10 @@
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="B234" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C234" t="s">
         <v>159</v>
@@ -5269,10 +5275,10 @@
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B235" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C235" t="s">
         <v>160</v>
@@ -5280,10 +5286,10 @@
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="B236" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C236" t="s">
         <v>161</v>
@@ -5291,21 +5297,21 @@
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="B237" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="C237" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="B238" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C238" t="s">
         <v>200</v>
@@ -5313,10 +5319,10 @@
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="B239" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="C239" t="s">
         <v>201</v>
@@ -5324,7 +5330,7 @@
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B240" t="s">
         <v>202</v>
@@ -5335,62 +5341,62 @@
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="B241" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C241" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="B242" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C242" t="s">
-        <v>204</v>
+        <v>413</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B243" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="C243" t="s">
-        <v>205</v>
+        <v>757</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B244" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="C244" t="s">
-        <v>204</v>
+        <v>413</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B245" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C245" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B246" t="s">
         <v>203</v>
@@ -5401,469 +5407,480 @@
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B247" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C247" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B248" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C248" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B249" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C249" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B250" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C250" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B251" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C251" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B252" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C252" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="B253" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C253" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B254" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C254" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="B255" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C255" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B256" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C256" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B257" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="C257" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B258" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C258" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="B259" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C259" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="B260" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C260" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="B261" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C261" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B262" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C262" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="B263" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C263" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="B264" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C264" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="B265" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C265" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="B266" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C266" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B267" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C267" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>665</v>
+        <v>758</v>
       </c>
       <c r="B268" t="s">
-        <v>434</v>
+        <v>759</v>
       </c>
       <c r="C268" t="s">
-        <v>231</v>
+        <v>760</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
       <c r="B269" t="s">
-        <v>423</v>
+        <v>432</v>
       </c>
       <c r="C269" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>721</v>
+        <v>653</v>
       </c>
       <c r="B270" t="s">
-        <v>709</v>
+        <v>421</v>
       </c>
       <c r="C270" t="s">
-        <v>733</v>
+        <v>220</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>657</v>
+        <v>719</v>
       </c>
       <c r="B271" t="s">
-        <v>425</v>
+        <v>707</v>
       </c>
       <c r="C271" t="s">
-        <v>223</v>
+        <v>731</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="B272" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="C272" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="B273" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="C273" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>663</v>
+        <v>658</v>
       </c>
       <c r="B274" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="C274" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>723</v>
+        <v>661</v>
       </c>
       <c r="B275" t="s">
-        <v>711</v>
+        <v>430</v>
       </c>
       <c r="C275" t="s">
-        <v>735</v>
+        <v>227</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>726</v>
+        <v>721</v>
       </c>
       <c r="B276" t="s">
-        <v>699</v>
+        <v>709</v>
       </c>
       <c r="C276" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>664</v>
+        <v>724</v>
       </c>
       <c r="B277" t="s">
-        <v>433</v>
+        <v>697</v>
       </c>
       <c r="C277" t="s">
-        <v>230</v>
+        <v>725</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
       <c r="B278" t="s">
-        <v>232</v>
+        <v>431</v>
       </c>
       <c r="C278" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="B279" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C279" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="B280" t="s">
-        <v>435</v>
+        <v>231</v>
       </c>
       <c r="C280" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="B281" t="s">
-        <v>670</v>
+        <v>433</v>
       </c>
       <c r="C281" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="B282" t="s">
-        <v>436</v>
+        <v>668</v>
       </c>
       <c r="C282" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="B283" t="s">
-        <v>237</v>
+        <v>434</v>
       </c>
       <c r="C283" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="B284" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C284" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="B285" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C285" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="B286" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C286" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="B287" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C287" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="B288" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C288" t="s">
-        <v>242</v>
+        <v>239</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>675</v>
+      </c>
+      <c r="B289" t="s">
+        <v>240</v>
+      </c>
+      <c r="C289" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C288">
-    <sortCondition ref="A2:A288"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C289">
+    <sortCondition ref="A2:A289"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Około 100 błędów w PNA
</commit_message>
<xml_diff>
--- a/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
+++ b/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\AddressLibrary\AddressLibrary\AppData\Dictionaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB331D2-911B-4F7B-AE19-50C0C303EAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE69C90-B24E-4B91-8DE3-6ECDBB87A8A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="761">
   <si>
     <t>abp</t>
   </si>
@@ -2691,7 +2691,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD74A5C-AF8A-492F-8246-0B7893A73121}">
-  <dimension ref="A1:C289"/>
+  <dimension ref="A1:C290"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" customWidth="1"/>
@@ -5878,6 +5878,17 @@
         <v>240</v>
       </c>
     </row>
+    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A290" t="s">
+        <v>639</v>
+      </c>
+      <c r="B290" t="s">
+        <v>204</v>
+      </c>
+      <c r="C290" t="s">
+        <v>204</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C289">
     <sortCondition ref="A2:A289"/>

</xml_diff>

<commit_message>
Wyczyszczone PNA i nowe TERYT - wszystko działa
</commit_message>
<xml_diff>
--- a/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
+++ b/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\AddressLibrary\AddressLibrary\AppData\Dictionaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5C10ED9-1133-4B52-B13D-B311C89D4750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995D3BC1-F5BB-4A44-AB51-117D57C10363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="768">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="773">
   <si>
     <t>abp</t>
   </si>
@@ -2340,6 +2340,21 @@
   </si>
   <si>
     <t xml:space="preserve">marsz. Rzeczpospolitej Polskiej </t>
+  </si>
+  <si>
+    <t>księdza doktora majora</t>
+  </si>
+  <si>
+    <t>hrabianki</t>
+  </si>
+  <si>
+    <t>ksiądz doktor major</t>
+  </si>
+  <si>
+    <t>hrabianka</t>
+  </si>
+  <si>
+    <t>ks. dr mjr</t>
   </si>
 </sst>
 </file>
@@ -2712,7 +2727,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD74A5C-AF8A-492F-8246-0B7893A73121}">
-  <dimension ref="A1:C294"/>
+  <dimension ref="A1:C296"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" customWidth="1"/>
@@ -5954,6 +5969,28 @@
         <v>240</v>
       </c>
     </row>
+    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A295" t="s">
+        <v>770</v>
+      </c>
+      <c r="B295" t="s">
+        <v>768</v>
+      </c>
+      <c r="C295" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
+        <v>771</v>
+      </c>
+      <c r="B296" t="s">
+        <v>769</v>
+      </c>
+      <c r="C296" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C294">
     <sortCondition ref="A2:A294"/>

</xml_diff>

<commit_message>
Wszystko sie ładuje, nowy Teryt ujarzmiony
</commit_message>
<xml_diff>
--- a/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
+++ b/AddressLibrary/AppData/Dictionaries/TytulyStopnie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\AddressLibrary\AddressLibrary\AppData\Dictionaries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995D3BC1-F5BB-4A44-AB51-117D57C10363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EEEFFE-5948-4689-8E92-DD3502E290CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
+    <workbookView xWindow="2940" yWindow="1455" windowWidth="21600" windowHeight="11295" xr2:uid="{64470E6A-0831-46D8-BC34-D7CB2F29E56A}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="773">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="903" uniqueCount="781">
   <si>
     <t>abp</t>
   </si>
@@ -2355,6 +2355,30 @@
   </si>
   <si>
     <t>ks. dr mjr</t>
+  </si>
+  <si>
+    <t>świętych braci</t>
+  </si>
+  <si>
+    <t>wojewody</t>
+  </si>
+  <si>
+    <t>świętego królewicza</t>
+  </si>
+  <si>
+    <t>prezydentów</t>
+  </si>
+  <si>
+    <t>ksieni</t>
+  </si>
+  <si>
+    <t>święci bracia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wojewoda </t>
+  </si>
+  <si>
+    <t>święty królewicz</t>
   </si>
 </sst>
 </file>
@@ -2727,7 +2751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BD74A5C-AF8A-492F-8246-0B7893A73121}">
-  <dimension ref="A1:C296"/>
+  <dimension ref="A1:C301"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.42578125" customWidth="1"/>
@@ -3518,10 +3542,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>688</v>
+        <v>771</v>
       </c>
       <c r="B72" t="s">
-        <v>678</v>
+        <v>769</v>
       </c>
       <c r="C72" t="s">
         <v>53</v>
@@ -3529,123 +3553,123 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>764</v>
+        <v>688</v>
       </c>
       <c r="B73" t="s">
-        <v>761</v>
+        <v>678</v>
       </c>
       <c r="C73" t="s">
-        <v>761</v>
+        <v>53</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>487</v>
+        <v>764</v>
       </c>
       <c r="B74" t="s">
-        <v>305</v>
+        <v>761</v>
       </c>
       <c r="C74" t="s">
-        <v>54</v>
+        <v>761</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B75" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C75" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B76" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C76" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B77" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C77" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B78" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C78" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="B79" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C79" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B80" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C80" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="B81" t="s">
-        <v>62</v>
+        <v>311</v>
       </c>
       <c r="C81" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B82" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C82" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>505</v>
+        <v>496</v>
       </c>
       <c r="B83" t="s">
-        <v>318</v>
+        <v>63</v>
       </c>
       <c r="C83" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -3653,7 +3677,7 @@
         <v>505</v>
       </c>
       <c r="B84" t="s">
-        <v>505</v>
+        <v>318</v>
       </c>
       <c r="C84" t="s">
         <v>72</v>
@@ -3661,178 +3685,178 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B85" t="s">
-        <v>319</v>
+        <v>505</v>
       </c>
       <c r="C85" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B86" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C86" t="s">
-        <v>738</v>
+        <v>73</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B87" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C87" t="s">
-        <v>74</v>
+        <v>738</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B88" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C88" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B89" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C89" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>503</v>
+        <v>510</v>
       </c>
       <c r="B90" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="C90" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B91" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C91" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
       <c r="B92" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C92" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>716</v>
+        <v>497</v>
       </c>
       <c r="B93" t="s">
-        <v>703</v>
+        <v>312</v>
       </c>
       <c r="C93" t="s">
-        <v>729</v>
+        <v>64</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>498</v>
+        <v>716</v>
       </c>
       <c r="B94" t="s">
-        <v>65</v>
+        <v>703</v>
       </c>
       <c r="C94" t="s">
-        <v>65</v>
+        <v>729</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>766</v>
+        <v>498</v>
       </c>
       <c r="B95" t="s">
-        <v>762</v>
+        <v>65</v>
       </c>
       <c r="C95" t="s">
-        <v>762</v>
+        <v>65</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>499</v>
+        <v>766</v>
       </c>
       <c r="B96" t="s">
-        <v>313</v>
+        <v>762</v>
       </c>
       <c r="C96" t="s">
-        <v>66</v>
+        <v>762</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B97" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C97" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B98" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C98" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="B99" t="s">
-        <v>69</v>
+        <v>314</v>
       </c>
       <c r="C99" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>492</v>
+        <v>502</v>
       </c>
       <c r="B100" t="s">
-        <v>492</v>
+        <v>69</v>
       </c>
       <c r="C100" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
@@ -3840,7 +3864,7 @@
         <v>492</v>
       </c>
       <c r="B101" t="s">
-        <v>679</v>
+        <v>492</v>
       </c>
       <c r="C101" t="s">
         <v>59</v>
@@ -3848,1913 +3872,1913 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>511</v>
+        <v>492</v>
       </c>
       <c r="B102" t="s">
-        <v>77</v>
+        <v>679</v>
       </c>
       <c r="C102" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B103" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C103" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B104" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C104" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B105" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C105" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B106" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C106" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>449</v>
+        <v>515</v>
       </c>
       <c r="B107" t="s">
-        <v>265</v>
+        <v>81</v>
       </c>
       <c r="C107" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>516</v>
+        <v>449</v>
       </c>
       <c r="B108" t="s">
-        <v>324</v>
+        <v>265</v>
       </c>
       <c r="C108" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B109" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C109" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B110" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C110" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B111" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C111" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B112" t="s">
-        <v>266</v>
+        <v>327</v>
       </c>
       <c r="C112" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>521</v>
+        <v>770</v>
       </c>
       <c r="B113" t="s">
-        <v>267</v>
+        <v>768</v>
       </c>
       <c r="C113" t="s">
-        <v>88</v>
+        <v>772</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="B114" t="s">
-        <v>328</v>
+        <v>266</v>
       </c>
       <c r="C114" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="B115" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C115" t="s">
-        <v>330</v>
+        <v>88</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="B116" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C116" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="B117" t="s">
-        <v>331</v>
+        <v>268</v>
       </c>
       <c r="C117" t="s">
-        <v>91</v>
+        <v>330</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="B118" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C118" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B119" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C119" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B120" t="s">
-        <v>269</v>
+        <v>333</v>
       </c>
       <c r="C120" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>713</v>
+        <v>526</v>
       </c>
       <c r="B121" t="s">
-        <v>700</v>
+        <v>332</v>
       </c>
       <c r="C121" t="s">
-        <v>727</v>
+        <v>92</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="B122" t="s">
-        <v>335</v>
+        <v>269</v>
       </c>
       <c r="C122" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>529</v>
+        <v>713</v>
       </c>
       <c r="B123" t="s">
-        <v>270</v>
+        <v>700</v>
       </c>
       <c r="C123" t="s">
-        <v>95</v>
+        <v>727</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B124" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C124" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="B125" t="s">
-        <v>337</v>
+        <v>270</v>
       </c>
       <c r="C125" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="B126" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C126" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>717</v>
+        <v>533</v>
       </c>
       <c r="B127" t="s">
-        <v>704</v>
+        <v>337</v>
       </c>
       <c r="C127" t="s">
-        <v>730</v>
+        <v>99</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="B128" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C128" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>537</v>
+        <v>717</v>
       </c>
       <c r="B129" t="s">
-        <v>341</v>
+        <v>704</v>
       </c>
       <c r="C129" t="s">
-        <v>103</v>
+        <v>730</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="B130" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C130" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B131" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C131" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="B132" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C132" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B133" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C133" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="B134" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C134" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B135" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C135" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B136" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C136" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B137" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C137" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="B138" t="s">
-        <v>546</v>
+        <v>347</v>
       </c>
       <c r="C138" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B139" t="s">
-        <v>685</v>
+        <v>348</v>
       </c>
       <c r="C139" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>535</v>
+        <v>545</v>
       </c>
       <c r="B140" t="s">
-        <v>339</v>
+        <v>546</v>
       </c>
       <c r="C140" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="B141" t="s">
-        <v>271</v>
+        <v>685</v>
       </c>
       <c r="C141" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>548</v>
+        <v>535</v>
       </c>
       <c r="B142" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="C142" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="B143" t="s">
-        <v>115</v>
+        <v>271</v>
       </c>
       <c r="C143" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B144" t="s">
-        <v>114</v>
+        <v>349</v>
       </c>
       <c r="C144" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>743</v>
+        <v>550</v>
       </c>
       <c r="B145" t="s">
-        <v>705</v>
+        <v>115</v>
       </c>
       <c r="C145" t="s">
-        <v>705</v>
+        <v>115</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B146" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C146" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>552</v>
+        <v>777</v>
       </c>
       <c r="B147" t="s">
-        <v>117</v>
+        <v>777</v>
       </c>
       <c r="C147" t="s">
-        <v>117</v>
+        <v>777</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>553</v>
+        <v>743</v>
       </c>
       <c r="B148" t="s">
-        <v>118</v>
+        <v>705</v>
       </c>
       <c r="C148" t="s">
-        <v>118</v>
+        <v>705</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="B149" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C149" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="B150" t="s">
-        <v>350</v>
+        <v>117</v>
       </c>
       <c r="C150" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="B151" t="s">
-        <v>351</v>
+        <v>118</v>
       </c>
       <c r="C151" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="B152" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C152" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>565</v>
+        <v>555</v>
       </c>
       <c r="B153" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="C153" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>566</v>
+        <v>556</v>
       </c>
       <c r="B154" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C154" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>569</v>
+        <v>557</v>
       </c>
       <c r="B155" t="s">
-        <v>357</v>
+        <v>122</v>
       </c>
       <c r="C155" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>570</v>
+        <v>565</v>
       </c>
       <c r="B156" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="C156" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>571</v>
+        <v>566</v>
       </c>
       <c r="B157" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="C157" t="s">
-        <v>744</v>
+        <v>131</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="B158" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="C158" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="B159" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="C159" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="B160" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C160" t="s">
-        <v>138</v>
+        <v>744</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>558</v>
+        <v>572</v>
       </c>
       <c r="B161" t="s">
-        <v>352</v>
+        <v>361</v>
       </c>
       <c r="C161" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>559</v>
+        <v>573</v>
       </c>
       <c r="B162" t="s">
-        <v>353</v>
+        <v>362</v>
       </c>
       <c r="C162" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>765</v>
+        <v>574</v>
       </c>
       <c r="B163" t="s">
-        <v>763</v>
+        <v>363</v>
       </c>
       <c r="C163" t="s">
-        <v>767</v>
+        <v>138</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B164" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="C164" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B165" t="s">
-        <v>126</v>
+        <v>353</v>
       </c>
       <c r="C165" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>562</v>
+        <v>765</v>
       </c>
       <c r="B166" t="s">
-        <v>127</v>
+        <v>763</v>
       </c>
       <c r="C166" t="s">
-        <v>127</v>
+        <v>767</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="B167" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C167" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="B168" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C168" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="B169" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C169" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="B170" t="s">
-        <v>133</v>
+        <v>354</v>
       </c>
       <c r="C170" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>575</v>
+        <v>564</v>
       </c>
       <c r="B171" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C171" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>712</v>
+        <v>567</v>
       </c>
       <c r="B172" t="s">
-        <v>699</v>
+        <v>132</v>
       </c>
       <c r="C172" t="s">
-        <v>726</v>
+        <v>132</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>715</v>
+        <v>568</v>
       </c>
       <c r="B173" t="s">
-        <v>702</v>
+        <v>133</v>
       </c>
       <c r="C173" t="s">
-        <v>726</v>
+        <v>133</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B174" t="s">
-        <v>364</v>
+        <v>139</v>
       </c>
       <c r="C174" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>577</v>
+        <v>712</v>
       </c>
       <c r="B175" t="s">
-        <v>365</v>
+        <v>699</v>
       </c>
       <c r="C175" t="s">
-        <v>141</v>
+        <v>726</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>578</v>
+        <v>715</v>
       </c>
       <c r="B176" t="s">
-        <v>366</v>
+        <v>702</v>
       </c>
       <c r="C176" t="s">
-        <v>142</v>
+        <v>726</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="B177" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C177" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="B178" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C178" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>714</v>
+        <v>578</v>
       </c>
       <c r="B179" t="s">
-        <v>701</v>
+        <v>366</v>
       </c>
       <c r="C179" t="s">
-        <v>728</v>
+        <v>142</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="B180" t="s">
-        <v>145</v>
+        <v>367</v>
       </c>
       <c r="C180" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B181" t="s">
-        <v>146</v>
+        <v>368</v>
       </c>
       <c r="C181" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>147</v>
+        <v>714</v>
       </c>
       <c r="B182" t="s">
-        <v>147</v>
+        <v>701</v>
       </c>
       <c r="C182" t="s">
-        <v>147</v>
+        <v>728</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B183" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C183" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B184" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C184" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>585</v>
+        <v>147</v>
       </c>
       <c r="B185" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C185" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="B186" t="s">
-        <v>371</v>
+        <v>148</v>
       </c>
       <c r="C186" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="B187" t="s">
-        <v>372</v>
+        <v>149</v>
       </c>
       <c r="C187" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>596</v>
+        <v>585</v>
       </c>
       <c r="B188" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="C188" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B189" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C189" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="B190" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C190" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B191" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C191" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>611</v>
+        <v>586</v>
       </c>
       <c r="B192" t="s">
-        <v>391</v>
+        <v>369</v>
       </c>
       <c r="C192" t="s">
-        <v>176</v>
+        <v>151</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>611</v>
+        <v>587</v>
       </c>
       <c r="B193" t="s">
-        <v>611</v>
+        <v>370</v>
       </c>
       <c r="C193" t="s">
-        <v>176</v>
+        <v>152</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>612</v>
+        <v>597</v>
       </c>
       <c r="B194" t="s">
-        <v>392</v>
+        <v>163</v>
       </c>
       <c r="C194" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="B195" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C195" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="B196" t="s">
-        <v>394</v>
+        <v>611</v>
       </c>
       <c r="C196" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="B197" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="C197" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
       <c r="B198" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="C198" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>607</v>
+        <v>614</v>
       </c>
       <c r="B199" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="C199" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>608</v>
+        <v>615</v>
       </c>
       <c r="B200" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C200" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="B201" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C201" t="s">
-        <v>389</v>
+        <v>172</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="B202" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="C202" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>598</v>
+        <v>608</v>
       </c>
       <c r="B203" t="s">
-        <v>164</v>
+        <v>387</v>
       </c>
       <c r="C203" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>599</v>
+        <v>609</v>
       </c>
       <c r="B204" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="C204" t="s">
-        <v>165</v>
+        <v>389</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>600</v>
+        <v>610</v>
       </c>
       <c r="B205" t="s">
-        <v>381</v>
+        <v>390</v>
       </c>
       <c r="C205" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="B206" t="s">
-        <v>382</v>
+        <v>164</v>
       </c>
       <c r="C206" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="B207" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="C207" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="B208" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="C208" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="B209" t="s">
-        <v>170</v>
+        <v>382</v>
       </c>
       <c r="C209" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="B210" t="s">
-        <v>171</v>
+        <v>383</v>
       </c>
       <c r="C210" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>616</v>
+        <v>603</v>
       </c>
       <c r="B211" t="s">
-        <v>182</v>
+        <v>384</v>
       </c>
       <c r="C211" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>617</v>
+        <v>604</v>
       </c>
       <c r="B212" t="s">
-        <v>397</v>
+        <v>170</v>
       </c>
       <c r="C212" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>618</v>
+        <v>605</v>
       </c>
       <c r="B213" t="s">
-        <v>396</v>
+        <v>171</v>
       </c>
       <c r="C213" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>756</v>
+        <v>616</v>
       </c>
       <c r="B214" t="s">
-        <v>755</v>
+        <v>182</v>
       </c>
       <c r="C214" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B215" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C215" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="B216" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="C216" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>720</v>
+        <v>756</v>
       </c>
       <c r="B217" t="s">
-        <v>708</v>
+        <v>755</v>
       </c>
       <c r="C217" t="s">
-        <v>732</v>
+        <v>187</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>621</v>
+        <v>756</v>
       </c>
       <c r="B218" t="s">
-        <v>400</v>
+        <v>776</v>
       </c>
       <c r="C218" t="s">
-        <v>187</v>
+        <v>776</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>745</v>
+        <v>619</v>
       </c>
       <c r="B219" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="C219" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B220" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="C220" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>623</v>
+        <v>720</v>
       </c>
       <c r="B221" t="s">
-        <v>403</v>
+        <v>708</v>
       </c>
       <c r="C221" t="s">
-        <v>190</v>
+        <v>732</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="B222" t="s">
-        <v>623</v>
+        <v>400</v>
       </c>
       <c r="C222" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>624</v>
+        <v>745</v>
       </c>
       <c r="B223" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="C223" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="B224" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="C224" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="B225" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="C225" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="B226" t="s">
-        <v>407</v>
+        <v>623</v>
       </c>
       <c r="C226" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>692</v>
+        <v>624</v>
       </c>
       <c r="B227" t="s">
-        <v>681</v>
+        <v>404</v>
       </c>
       <c r="C227" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="B228" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C228" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>746</v>
+        <v>626</v>
       </c>
       <c r="B229" t="s">
-        <v>748</v>
+        <v>406</v>
       </c>
       <c r="C229" t="s">
-        <v>750</v>
+        <v>193</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>747</v>
+        <v>627</v>
       </c>
       <c r="B230" t="s">
-        <v>749</v>
+        <v>407</v>
       </c>
       <c r="C230" t="s">
-        <v>751</v>
+        <v>194</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>629</v>
+        <v>692</v>
       </c>
       <c r="B231" t="s">
-        <v>409</v>
+        <v>681</v>
       </c>
       <c r="C231" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B232" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C232" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>631</v>
+        <v>746</v>
       </c>
       <c r="B233" t="s">
-        <v>198</v>
+        <v>748</v>
       </c>
       <c r="C233" t="s">
-        <v>198</v>
+        <v>750</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>632</v>
+        <v>747</v>
       </c>
       <c r="B234" t="s">
-        <v>199</v>
+        <v>749</v>
       </c>
       <c r="C234" t="s">
-        <v>199</v>
+        <v>751</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>590</v>
+        <v>629</v>
       </c>
       <c r="B235" t="s">
-        <v>373</v>
+        <v>409</v>
       </c>
       <c r="C235" t="s">
-        <v>155</v>
+        <v>196</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>591</v>
+        <v>630</v>
       </c>
       <c r="B236" t="s">
-        <v>374</v>
+        <v>410</v>
       </c>
       <c r="C236" t="s">
-        <v>156</v>
+        <v>197</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>592</v>
+        <v>631</v>
       </c>
       <c r="B237" t="s">
-        <v>375</v>
+        <v>198</v>
       </c>
       <c r="C237" t="s">
-        <v>157</v>
+        <v>198</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>593</v>
+        <v>632</v>
       </c>
       <c r="B238" t="s">
-        <v>376</v>
+        <v>199</v>
       </c>
       <c r="C238" t="s">
-        <v>158</v>
+        <v>199</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="B239" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="C239" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="B240" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C240" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>752</v>
+        <v>592</v>
       </c>
       <c r="B241" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C241" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>722</v>
+        <v>593</v>
       </c>
       <c r="B242" t="s">
-        <v>711</v>
+        <v>376</v>
       </c>
       <c r="C242" t="s">
-        <v>711</v>
+        <v>158</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>633</v>
+        <v>594</v>
       </c>
       <c r="B243" t="s">
-        <v>411</v>
+        <v>377</v>
       </c>
       <c r="C243" t="s">
-        <v>200</v>
+        <v>159</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>634</v>
+        <v>595</v>
       </c>
       <c r="B244" t="s">
-        <v>412</v>
+        <v>378</v>
       </c>
       <c r="C244" t="s">
-        <v>201</v>
+        <v>160</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>635</v>
+        <v>752</v>
       </c>
       <c r="B245" t="s">
-        <v>202</v>
+        <v>379</v>
       </c>
       <c r="C245" t="s">
-        <v>202</v>
+        <v>161</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>639</v>
+        <v>722</v>
       </c>
       <c r="B246" t="s">
-        <v>204</v>
+        <v>711</v>
       </c>
       <c r="C246" t="s">
-        <v>204</v>
+        <v>711</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
       <c r="B247" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C247" t="s">
-        <v>413</v>
+        <v>200</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="B248" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="C248" t="s">
-        <v>757</v>
+        <v>201</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>413</v>
+        <v>635</v>
       </c>
       <c r="B249" t="s">
-        <v>710</v>
+        <v>202</v>
       </c>
       <c r="C249" t="s">
-        <v>413</v>
+        <v>202</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B250" t="s">
-        <v>415</v>
+        <v>204</v>
       </c>
       <c r="C250" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B251" t="s">
-        <v>203</v>
+        <v>413</v>
       </c>
       <c r="C251" t="s">
-        <v>203</v>
+        <v>413</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B252" t="s">
-        <v>206</v>
+        <v>414</v>
       </c>
       <c r="C252" t="s">
-        <v>206</v>
+        <v>757</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>642</v>
+        <v>413</v>
       </c>
       <c r="B253" t="s">
-        <v>207</v>
+        <v>710</v>
       </c>
       <c r="C253" t="s">
-        <v>207</v>
+        <v>413</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="B254" t="s">
-        <v>209</v>
+        <v>415</v>
       </c>
       <c r="C254" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>210</v>
+        <v>636</v>
       </c>
       <c r="B255" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="C255" t="s">
-        <v>694</v>
+        <v>203</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>210</v>
+        <v>641</v>
       </c>
       <c r="B256" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C256" t="s">
-        <v>694</v>
+        <v>206</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="B257" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C257" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B258" t="s">
-        <v>417</v>
+        <v>209</v>
       </c>
       <c r="C258" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>647</v>
+        <v>210</v>
       </c>
       <c r="B259" t="s">
-        <v>418</v>
+        <v>211</v>
       </c>
       <c r="C259" t="s">
-        <v>214</v>
+        <v>694</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>648</v>
+        <v>210</v>
       </c>
       <c r="B260" t="s">
-        <v>419</v>
+        <v>210</v>
       </c>
       <c r="C260" t="s">
-        <v>215</v>
+        <v>694</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B261" t="s">
-        <v>416</v>
+        <v>212</v>
       </c>
       <c r="C261" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>416</v>
+        <v>646</v>
       </c>
       <c r="B262" t="s">
-        <v>696</v>
+        <v>417</v>
       </c>
       <c r="C262" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>216</v>
+        <v>647</v>
       </c>
       <c r="B263" t="s">
-        <v>216</v>
+        <v>418</v>
       </c>
       <c r="C263" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>718</v>
+        <v>648</v>
       </c>
       <c r="B264" t="s">
-        <v>706</v>
+        <v>419</v>
       </c>
       <c r="C264" t="s">
-        <v>706</v>
+        <v>215</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="B265" t="s">
-        <v>218</v>
+        <v>416</v>
       </c>
       <c r="C265" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>651</v>
+        <v>416</v>
       </c>
       <c r="B266" t="s">
-        <v>219</v>
+        <v>696</v>
       </c>
       <c r="C266" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>649</v>
+        <v>216</v>
       </c>
       <c r="B267" t="s">
-        <v>420</v>
+        <v>216</v>
       </c>
       <c r="C267" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>654</v>
+        <v>718</v>
       </c>
       <c r="B268" t="s">
-        <v>426</v>
+        <v>706</v>
       </c>
       <c r="C268" t="s">
-        <v>220</v>
+        <v>706</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>656</v>
+        <v>650</v>
       </c>
       <c r="B269" t="s">
-        <v>424</v>
+        <v>218</v>
       </c>
       <c r="C269" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B270" t="s">
-        <v>422</v>
+        <v>219</v>
       </c>
       <c r="C270" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>659</v>
+        <v>649</v>
       </c>
       <c r="B271" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
       <c r="C271" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>660</v>
+        <v>654</v>
       </c>
       <c r="B272" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="C272" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>758</v>
+        <v>656</v>
       </c>
       <c r="B273" t="s">
-        <v>759</v>
+        <v>424</v>
       </c>
       <c r="C273" t="s">
-        <v>760</v>
+        <v>222</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>663</v>
+        <v>778</v>
       </c>
       <c r="B274" t="s">
-        <v>432</v>
+        <v>773</v>
       </c>
       <c r="C274" t="s">
-        <v>229</v>
+        <v>773</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B275" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C275" t="s">
         <v>220</v>
@@ -5762,238 +5786,293 @@
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>719</v>
+        <v>659</v>
       </c>
       <c r="B276" t="s">
-        <v>707</v>
+        <v>428</v>
       </c>
       <c r="C276" t="s">
-        <v>731</v>
+        <v>225</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="B277" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="C277" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>657</v>
+        <v>758</v>
       </c>
       <c r="B278" t="s">
-        <v>425</v>
+        <v>759</v>
       </c>
       <c r="C278" t="s">
-        <v>223</v>
+        <v>760</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="B279" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="C279" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>661</v>
+        <v>653</v>
       </c>
       <c r="B280" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="C280" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="B281" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="C281" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>724</v>
+        <v>655</v>
       </c>
       <c r="B282" t="s">
-        <v>697</v>
+        <v>423</v>
       </c>
       <c r="C282" t="s">
-        <v>725</v>
+        <v>221</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>662</v>
+        <v>657</v>
       </c>
       <c r="B283" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="C283" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>664</v>
+        <v>658</v>
       </c>
       <c r="B284" t="s">
-        <v>230</v>
+        <v>427</v>
       </c>
       <c r="C284" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>665</v>
+        <v>780</v>
       </c>
       <c r="B285" t="s">
-        <v>231</v>
+        <v>775</v>
       </c>
       <c r="C285" t="s">
-        <v>231</v>
+        <v>775</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>666</v>
+        <v>661</v>
       </c>
       <c r="B286" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="C286" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>667</v>
+        <v>721</v>
       </c>
       <c r="B287" t="s">
-        <v>668</v>
+        <v>709</v>
       </c>
       <c r="C287" t="s">
-        <v>233</v>
+        <v>733</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>669</v>
+        <v>724</v>
       </c>
       <c r="B288" t="s">
-        <v>434</v>
+        <v>697</v>
       </c>
       <c r="C288" t="s">
-        <v>234</v>
+        <v>725</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>670</v>
+        <v>662</v>
       </c>
       <c r="B289" t="s">
-        <v>235</v>
+        <v>431</v>
       </c>
       <c r="C289" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>671</v>
+        <v>664</v>
       </c>
       <c r="B290" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="C290" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>672</v>
+        <v>665</v>
       </c>
       <c r="B291" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="C291" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>673</v>
+        <v>666</v>
       </c>
       <c r="B292" t="s">
-        <v>238</v>
+        <v>433</v>
       </c>
       <c r="C292" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>674</v>
+        <v>667</v>
       </c>
       <c r="B293" t="s">
-        <v>239</v>
+        <v>668</v>
       </c>
       <c r="C293" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="294" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="B294" t="s">
-        <v>240</v>
+        <v>434</v>
       </c>
       <c r="C294" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>770</v>
+        <v>670</v>
       </c>
       <c r="B295" t="s">
-        <v>768</v>
+        <v>235</v>
       </c>
       <c r="C295" t="s">
-        <v>772</v>
+        <v>235</v>
       </c>
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>771</v>
+        <v>671</v>
       </c>
       <c r="B296" t="s">
-        <v>769</v>
+        <v>236</v>
       </c>
       <c r="C296" t="s">
-        <v>53</v>
+        <v>236</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A297" t="s">
+        <v>779</v>
+      </c>
+      <c r="B297" t="s">
+        <v>774</v>
+      </c>
+      <c r="C297" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A298" t="s">
+        <v>672</v>
+      </c>
+      <c r="B298" t="s">
+        <v>237</v>
+      </c>
+      <c r="C298" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A299" t="s">
+        <v>673</v>
+      </c>
+      <c r="B299" t="s">
+        <v>238</v>
+      </c>
+      <c r="C299" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A300" t="s">
+        <v>674</v>
+      </c>
+      <c r="B300" t="s">
+        <v>239</v>
+      </c>
+      <c r="C300" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A301" t="s">
+        <v>675</v>
+      </c>
+      <c r="B301" t="s">
+        <v>240</v>
+      </c>
+      <c r="C301" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C294">
-    <sortCondition ref="A2:A294"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C301">
+    <sortCondition ref="A2:A301"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>